<commit_message>
Record admission evidence and preserve scoped feature verdicts
</commit_message>
<xml_diff>
--- a/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
+++ b/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
@@ -188,9 +188,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AvenFeatures" displayName="AvenFeatures" ref="A10:P125" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A10:P125"/>
-  <x:tableColumns count="16">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AvenFeatures" displayName="AvenFeatures" ref="A10:S125" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A10:S125"/>
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
     <x:tableColumn id="3" name="Feature"/>
@@ -207,6 +207,9 @@
     <x:tableColumn id="14" name="Delivery"/>
     <x:tableColumn id="15" name="Decision"/>
     <x:tableColumn id="16" name="Evidence"/>
+    <x:tableColumn id="17" name="Effective verdict 2026-09-19"/>
+    <x:tableColumn id="18" name="Admission evidence 2026-09-19"/>
+    <x:tableColumn id="19" name="Remaining scope / limits"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -404,7 +407,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF253448"/>
   </x:sheetPr>
@@ -426,6 +429,9 @@
     <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="46" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="29" customWidth="1"/>
+    <x:col min="18" max="18" width="72" customWidth="1"/>
+    <x:col min="19" max="19" width="65" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -651,7 +657,9 @@
       <x:c r="T8" s="1"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="1"/>
+      <x:c r="A9" s="1" t="str">
+        <x:v>19 September 2026: Q–S contain effective scoped verdicts and admission evidence. A–P and the summary above remain dated history. Counts: 37 scoped Verified, 57 Partial, 3 Unverified, 14 Missing, 4 Deferred; owner approval is separate.</x:v>
+      </x:c>
       <x:c r="B9" s="1"/>
       <x:c r="C9" s="1"/>
       <x:c r="D9" s="1"/>
@@ -721,9 +729,15 @@
       <x:c r="P10" s="8" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="Q10" s="1"/>
-      <x:c r="R10" s="1"/>
-      <x:c r="S10" s="1"/>
+      <x:c r="Q10" s="8" t="str">
+        <x:v>Effective verdict 2026-09-19</x:v>
+      </x:c>
+      <x:c r="R10" s="8" t="str">
+        <x:v>Admission evidence 2026-09-19</x:v>
+      </x:c>
+      <x:c r="S10" s="8" t="str">
+        <x:v>Remaining scope / limits</x:v>
+      </x:c>
       <x:c r="T10" s="1"/>
     </x:row>
     <x:row r="11" ht="117" customHeight="1">
@@ -775,9 +789,15 @@
       <x:c r="P11" s="15" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q11" s="1"/>
-      <x:c r="R11" s="1"/>
-      <x:c r="S11" s="1"/>
+      <x:c r="Q11" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R11" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S11" s="15" t="str">
+        <x:v>No substantive gap in the original browser interaction slice; assistive-technology and owner visual certification remain outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T11" s="1"/>
     </x:row>
     <x:row r="12" ht="117" customHeight="1">
@@ -829,9 +849,15 @@
       <x:c r="P12" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q12" s="1"/>
-      <x:c r="R12" s="1"/>
-      <x:c r="S12" s="1"/>
+      <x:c r="Q12" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R12" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S12" s="17" t="str">
+        <x:v>Agreed desktop-width matrix beyond 390px is untested, so full overflow coverage is incomplete. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T12" s="1"/>
     </x:row>
     <x:row r="13" ht="102" customHeight="1">
@@ -883,9 +909,15 @@
       <x:c r="P13" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/root-identity-review.json; review-ux-pipeline.cjs --identity-only; exit 0. Isolated Chromium, owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q13" s="1"/>
-      <x:c r="R13" s="1"/>
-      <x:c r="S13" s="1"/>
+      <x:c r="Q13" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R13" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S13" s="19" t="str">
+        <x:v>No substantive gap in the original browser interaction slice; assistive-technology certification remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T13" s="1"/>
     </x:row>
     <x:row r="14" ht="87" customHeight="1">
@@ -937,9 +969,15 @@
       <x:c r="P14" s="17" t="str">
         <x:v>2026-09-15: root-identity-review.json and root-profile-desktop.png under .intentgraph/evidence/ux-fixes-2026-09-15/; browser test exit 0. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q14" s="1"/>
-      <x:c r="R14" s="1"/>
-      <x:c r="S14" s="1"/>
+      <x:c r="Q14" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R14" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S14" s="17" t="str">
+        <x:v>The evidence does not open and edit every selected profile document after rename, so document accessibility is incomplete. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T14" s="1"/>
     </x:row>
     <x:row r="15" ht="117" customHeight="1">
@@ -991,9 +1029,15 @@
       <x:c r="P15" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q15" s="1"/>
-      <x:c r="R15" s="1"/>
-      <x:c r="S15" s="1"/>
+      <x:c r="Q15" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R15" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S15" s="19" t="str">
+        <x:v>Pointer/keyboard operation and bounds pass, but row structure has no current/reference visual or structural comparison. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T15" s="1"/>
     </x:row>
     <x:row r="16" ht="117" customHeight="1">
@@ -1045,9 +1089,15 @@
       <x:c r="P16" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q16" s="1"/>
-      <x:c r="R16" s="1"/>
-      <x:c r="S16" s="1"/>
+      <x:c r="Q16" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R16" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S16" s="17" t="str">
+        <x:v>No substantive gap in the original local interaction slice; concurrent-device synchronization remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T16" s="1"/>
     </x:row>
     <x:row r="17" ht="117" customHeight="1">
@@ -1099,9 +1149,15 @@
       <x:c r="P17" s="15" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q17" s="1"/>
-      <x:c r="R17" s="1"/>
-      <x:c r="S17" s="1"/>
+      <x:c r="Q17" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R17" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S17" s="15" t="str">
+        <x:v>The seeded test proves direct/grouped history, queue and avatar reachability, but does not exercise a new-user named-conversation start path. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T17" s="1"/>
     </x:row>
     <x:row r="18" ht="117" customHeight="1">
@@ -1153,9 +1209,15 @@
       <x:c r="P18" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-fixes-2026-09-15/history-regression.json (stable coworker title after hi); .intentgraph/runtime/verify-direct-teams.cjs:8,12 Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q18" s="1"/>
-      <x:c r="R18" s="1"/>
-      <x:c r="S18" s="1"/>
+      <x:c r="Q18" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R18" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S18" s="17" t="str">
+        <x:v>No substantive gap in the original UI identity slice; the provider stream is intentionally mocked/blocked. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T18" s="1"/>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
@@ -1207,9 +1269,15 @@
       <x:c r="P19" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/local-commands.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q19" s="1"/>
-      <x:c r="R19" s="1"/>
-      <x:c r="S19" s="1"/>
+      <x:c r="Q19" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R19" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S19" s="19" t="str">
+        <x:v>No substantive gap in the tested acceptance slice; only the seeded narrow width and title matrix were exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T19" s="1"/>
     </x:row>
     <x:row r="20" ht="72" customHeight="1">
@@ -1261,9 +1329,15 @@
       <x:c r="P20" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/project-navigation.json (pin/reload/order) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q20" s="1"/>
-      <x:c r="R20" s="1"/>
-      <x:c r="S20" s="1"/>
+      <x:c r="Q20" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R20" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S20" s="17" t="str">
+        <x:v>No substantive gap in the original local persistence slice; cross-device ordering remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T20" s="1"/>
     </x:row>
     <x:row r="21" ht="102" customHeight="1">
@@ -1315,9 +1389,15 @@
       <x:c r="P21" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (chatTitle changed; coworkerName unchanged) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q21" s="1"/>
-      <x:c r="R21" s="1"/>
-      <x:c r="S21" s="1"/>
+      <x:c r="Q21" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R21" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S21" s="19" t="str">
+        <x:v>No substantive gap in the original direct-conversation slice; broader multi-user synchronization remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T21" s="1"/>
     </x:row>
     <x:row r="22" ht="102" customHeight="1">
@@ -1369,9 +1449,15 @@
       <x:c r="P22" s="17" t="str">
         <x:v>2026-09-16: navigation.json; isolated browser test exit 0. Section boundaries, reload, failed-save atomicity and focus verified. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q22" s="1"/>
-      <x:c r="R22" s="1"/>
-      <x:c r="S22" s="1"/>
+      <x:c r="Q22" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R22" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S22" s="17" t="str">
+        <x:v>DOM separation and old-row reachability pass, but the evidence does not assert labels/affordances cannot imply coordinated execution. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T22" s="1"/>
     </x:row>
     <x:row r="23" ht="132" customHeight="1">
@@ -1423,9 +1509,15 @@
       <x:c r="P23" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/accessibility-results.json (UX096 PASS at 320/390/760/1440; page/body bounds); .intentgraph/evidence/project-navigation.json (persistent collapse) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q23" s="1"/>
-      <x:c r="R23" s="1"/>
-      <x:c r="S23" s="1"/>
+      <x:c r="Q23" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R23" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S23" s="19" t="str">
+        <x:v>No substantive gap in the original browser slice; assistive-technology certification remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T23" s="1"/>
     </x:row>
     <x:row r="24" ht="102" customHeight="1">
@@ -1477,9 +1569,15 @@
       <x:c r="P24" s="17" t="str">
         <x:v>2026-09-16: navigation.json; isolated browser test exit 0. Draft/scroll, reload, forward history, invalid storage, unsaved guards and 320-1440px bounds verified. No provider calls. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q24" s="1"/>
-      <x:c r="R24" s="1"/>
-      <x:c r="S24" s="1"/>
+      <x:c r="Q24" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R24" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S24" s="17" t="str">
+        <x:v>No substantive gap in the tested local session-history slice; cross-session/device history is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T24" s="1"/>
     </x:row>
     <x:row r="25" ht="117" customHeight="1">
@@ -1531,9 +1629,15 @@
       <x:c r="P25" s="15" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json (saved phrase, coworker/conversation filters, exact result navigation) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q25" s="1"/>
-      <x:c r="R25" s="1"/>
-      <x:c r="S25" s="1"/>
+      <x:c r="Q25" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R25" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S25" s="15" t="str">
+        <x:v>No substantive gap for the seeded known phrase; search-index breadth beyond local fixture data is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T25" s="1"/>
     </x:row>
     <x:row r="26" ht="87" customHeight="1">
@@ -1585,9 +1689,15 @@
       <x:c r="P26" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json; verify-history-navigation.cjs exit 0. Isolated mocked chat; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q26" s="1"/>
-      <x:c r="R26" s="1"/>
-      <x:c r="S26" s="1"/>
+      <x:c r="Q26" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R26" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S26" s="17" t="str">
+        <x:v>No substantive gap for the seeded duplicate-term filter result; broader external-index behavior is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T26" s="1"/>
     </x:row>
     <x:row r="27" ht="87" customHeight="1">
@@ -1639,9 +1749,15 @@
       <x:c r="P27" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/chat-interactions.json; verify-chat-interactions.cjs exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q27" s="1"/>
-      <x:c r="R27" s="1"/>
-      <x:c r="S27" s="1"/>
+      <x:c r="Q27" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R27" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S27" s="19" t="str">
+        <x:v>No substantive gap for the seeded repeated-term cycle; cross-conversation find scope is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T27" s="1"/>
     </x:row>
     <x:row r="28" ht="72" customHeight="1">
@@ -1693,9 +1809,15 @@
       <x:c r="P28" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/local-commands.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q28" s="1"/>
-      <x:c r="R28" s="1"/>
-      <x:c r="S28" s="1"/>
+      <x:c r="Q28" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R28" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S28" s="17" t="str">
+        <x:v>No substantive gap in the tested current-chat palette flow; OS-level shortcut conflicts remain outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T28" s="1"/>
     </x:row>
     <x:row r="29" ht="102" customHeight="1">
@@ -1747,9 +1869,15 @@
       <x:c r="P29" s="15" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (emptyDisabled=true, multilineHeld=true, imeHeld=true, calls=0) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q29" s="1"/>
-      <x:c r="R29" s="1"/>
-      <x:c r="S29" s="1"/>
+      <x:c r="Q29" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R29" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S29" s="15" t="str">
+        <x:v>IME composition was not simulated. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T29" s="1"/>
     </x:row>
     <x:row r="30" ht="102" customHeight="1">
@@ -1801,9 +1929,15 @@
       <x:c r="P30" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-pipeline-2026-09-16/navigation.json (back/forward preserves two drafts and reload) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q30" s="1"/>
-      <x:c r="R30" s="1"/>
-      <x:c r="S30" s="1"/>
+      <x:c r="Q30" s="17" t="str">
+        <x:v>Unverified</x:v>
+      </x:c>
+      <x:c r="R30" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S30" s="17" t="str">
+        <x:v>No fresh end-to-end evidence for independent drafts. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T30" s="1"/>
     </x:row>
     <x:row r="31" ht="102" customHeight="1">
@@ -1855,9 +1989,15 @@
       <x:c r="P31" s="19" t="str">
         <x:v>2026-09-16: attachments.json; verify-attachments-unit.cjs. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q31" s="1"/>
-      <x:c r="R31" s="1"/>
-      <x:c r="S31" s="1"/>
+      <x:c r="Q31" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R31" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S31" s="19" t="str">
+        <x:v>Fresh check did not inspect request context or unsupported-file pre-send behavior. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T31" s="1"/>
     </x:row>
     <x:row r="32" ht="72" customHeight="1">
@@ -1909,9 +2049,15 @@
       <x:c r="P32" s="17" t="str">
         <x:v>2026-09-16: attachments.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q32" s="1"/>
-      <x:c r="R32" s="1"/>
-      <x:c r="S32" s="1"/>
+      <x:c r="Q32" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R32" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S32" s="17" t="str">
+        <x:v>Drag/drop and clipboard paths were not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T32" s="1"/>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
@@ -1963,9 +2109,15 @@
       <x:c r="P33" s="19" t="str">
         <x:v>polished.html; polished.js; polished.js:213-265,408-437</x:v>
       </x:c>
-      <x:c r="Q33" s="1"/>
-      <x:c r="R33" s="1"/>
-      <x:c r="S33" s="1"/>
+      <x:c r="Q33" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R33" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S33" s="19" t="str">
+        <x:v>No provider, device, or credential calls were made by this audit. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T33" s="1"/>
     </x:row>
     <x:row r="34" ht="87" customHeight="1">
@@ -2017,9 +2169,15 @@
       <x:c r="P34" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/chat-interactions.json; verify-chat-interactions.cjs exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q34" s="1"/>
-      <x:c r="R34" s="1"/>
-      <x:c r="S34" s="1"/>
+      <x:c r="Q34" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R34" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S34" s="17" t="str">
+        <x:v>No substantive gap in the tested reply/cancel flow; the fixture used a mouse path only. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T34" s="1"/>
     </x:row>
     <x:row r="35" ht="72" customHeight="1">
@@ -2071,9 +2229,15 @@
       <x:c r="P35" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/edit-rendering.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q35" s="1"/>
-      <x:c r="R35" s="1"/>
-      <x:c r="S35" s="1"/>
+      <x:c r="Q35" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R35" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S35" s="19" t="str">
+        <x:v>No device command execution was permitted or tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T35" s="1"/>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
@@ -2125,9 +2289,15 @@
       <x:c r="P36" s="17" t="str">
         <x:v>polished.html composer; polished.js:213-265,408-437</x:v>
       </x:c>
-      <x:c r="Q36" s="1"/>
-      <x:c r="R36" s="1"/>
-      <x:c r="S36" s="1"/>
+      <x:c r="Q36" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R36" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S36" s="17" t="str">
+        <x:v>Microphone/device APIs were intentionally not called. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T36" s="1"/>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
@@ -2179,9 +2349,15 @@
       <x:c r="P37" s="19" t="str">
         <x:v>A0 Settings Models; agent-runtime.cjs; polished.js:213-265,408-437</x:v>
       </x:c>
-      <x:c r="Q37" s="1"/>
-      <x:c r="R37" s="1"/>
-      <x:c r="S37" s="1"/>
+      <x:c r="Q37" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R37" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S37" s="19" t="str">
+        <x:v>No real provider call was attempted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T37" s="1"/>
     </x:row>
     <x:row r="38" ht="117" customHeight="1">
@@ -2233,9 +2409,15 @@
       <x:c r="P38" s="21" t="str">
         <x:v>2026-09-16: preservation audit PASS. isolated run `node .intentgraph/runtime/verify-agent-stream-ui.cjs`; .intentgraph/evidence/chat-polish.json (one terminal despite duplicate event/final) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q38" s="1"/>
-      <x:c r="R38" s="1"/>
-      <x:c r="S38" s="1"/>
+      <x:c r="Q38" s="21" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R38" s="21" t="str">
+        <x:v>Current API and browser reconcile one final result after lost response/reload; exact 15-line code remains collapsed and intact. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S38" s="21" t="str">
+        <x:v>The stream was locally fulfilled; provider behavior and reconnects were not tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T38" s="1"/>
     </x:row>
     <x:row r="39" ht="87" customHeight="1">
@@ -2287,9 +2469,15 @@
       <x:c r="P39" s="19" t="str">
         <x:v>2026-09-16: verify-queue-terminal.cjs 4/4; run-durability.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q39" s="1"/>
-      <x:c r="R39" s="1"/>
-      <x:c r="S39" s="1"/>
+      <x:c r="Q39" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R39" s="19" t="str">
+        <x:v>Current Stop fixture preserves UNKNOWN and pauses queued work. Remote cancellation is not asserted. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S39" s="19" t="str">
+        <x:v>No real remote request or device command was stopped. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T39" s="1"/>
     </x:row>
     <x:row r="40" ht="132" customHeight="1">
@@ -2341,9 +2529,15 @@
       <x:c r="P40" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (storage failure: 0 calls, queue retained; recovery: 1 call); .intentgraph/runtime/verify-queue-terminal.cjs:49-75 Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q40" s="1"/>
-      <x:c r="R40" s="1"/>
-      <x:c r="S40" s="1"/>
+      <x:c r="Q40" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R40" s="17" t="str">
+        <x:v>Stable saved identities and backend duplicate suppression; current browser FIFO and explicit paused-queue checks. Broader crash-at-every-queue-boundary coverage remains partial. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S40" s="17" t="str">
+        <x:v>Order and duplicate-submission behavior were not freshly exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T40" s="1"/>
     </x:row>
     <x:row r="41" ht="87" customHeight="1">
@@ -2395,9 +2589,15 @@
       <x:c r="P41" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/runtime/verify-queue-terminal.cjs:49-75,120-128 (FIFO/edit/remove/resume/reload pause) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q41" s="1"/>
-      <x:c r="R41" s="1"/>
-      <x:c r="S41" s="1"/>
+      <x:c r="Q41" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R41" s="19" t="str">
+        <x:v>Current queue survives Stop/review and resumes explicitly; this milestone does not freshly exercise every edit/remove/reorder variant. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S41" s="19" t="str">
+        <x:v>Resume and exactly-once dispatch were not tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T41" s="1"/>
     </x:row>
     <x:row r="42" ht="132" customHeight="1">
@@ -2449,9 +2649,15 @@
       <x:c r="P42" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. 25/25 local fixture tests passed, including `intentgraph/steering.test.cjs:166-191` (next model boundary, applied once); .intentgraph/runtime/verify-queue-terminal.cjs:77-118 Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q42" s="1"/>
-      <x:c r="R42" s="1"/>
-      <x:c r="S42" s="1"/>
+      <x:c r="Q42" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R42" s="17" t="str">
+        <x:v>Existing active steering tests pass unchanged; receipt identity does not replace steering tokens or authorize new work. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S42" s="17" t="str">
+        <x:v>Unit coverage does not prove the browser UI flow. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T42" s="1"/>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
@@ -2503,9 +2709,15 @@
       <x:c r="P43" s="19" t="str">
         <x:v>A0; server/runtime source review; polished.js:193-255,380-422; intentgraph/server.cjs:206-285</x:v>
       </x:c>
-      <x:c r="Q43" s="1"/>
-      <x:c r="R43" s="1"/>
-      <x:c r="S43" s="1"/>
+      <x:c r="Q43" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R43" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S43" s="19" t="str">
+        <x:v>No external approval or device action was invoked. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T43" s="1"/>
     </x:row>
     <x:row r="44" ht="87" customHeight="1">
@@ -2557,9 +2769,15 @@
       <x:c r="P44" s="17" t="str">
         <x:v>2026-09-16: verify-chat-modes.cjs and modes-ui.json passed; malicious tool-call fixture invokes no sandbox. No live provider call.</x:v>
       </x:c>
-      <x:c r="Q44" s="1"/>
-      <x:c r="R44" s="1"/>
-      <x:c r="S44" s="1"/>
+      <x:c r="Q44" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R44" s="17" t="str">
+        <x:v>Existing Plan/Inspect and allowlist tests pass; browser Plan fixture uses the same saved mode on retries. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S44" s="17" t="str">
+        <x:v>The current fixture did not prove backend no-tools enforcement for every plan request. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T44" s="1"/>
     </x:row>
     <x:row r="45" ht="102" customHeight="1">
@@ -2611,9 +2829,15 @@
       <x:c r="P45" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/runtime/verify-queue-terminal.cjs:77-118 (tool input/result/status/raw output distinct); isolated stream UI passed Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q45" s="1"/>
-      <x:c r="R45" s="1"/>
-      <x:c r="S45" s="1"/>
+      <x:c r="Q45" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R45" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S45" s="19" t="str">
+        <x:v>No substantive gap in the saved transcript representation; provider-stream coverage remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T45" s="1"/>
     </x:row>
     <x:row r="46" ht="87" customHeight="1">
@@ -2665,9 +2889,15 @@
       <x:c r="P46" s="17" t="str">
         <x:v>2026-09-16: run-recovery.json; run-durability.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q46" s="1"/>
-      <x:c r="R46" s="1"/>
-      <x:c r="S46" s="1"/>
+      <x:c r="Q46" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R46" s="17" t="str">
+        <x:v>Unknown/cancellation/persistence failures cannot be promoted to success; elapsed UI behavior retains existing implementation. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S46" s="17" t="str">
+        <x:v>Elapsed timing itself was not asserted by the fresh harness. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T46" s="1"/>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
@@ -2719,9 +2949,15 @@
       <x:c r="P47" s="19" t="str">
         <x:v>server.cjs chatPending; architecture.json; polished.js:193-255,380-422; intentgraph/server.cjs:206-285</x:v>
       </x:c>
-      <x:c r="Q47" s="1"/>
-      <x:c r="R47" s="1"/>
-      <x:c r="S47" s="1"/>
+      <x:c r="Q47" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R47" s="19" t="str">
+        <x:v>Global serial admission retained. Parallel execution remains Missing. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S47" s="19" t="str">
+        <x:v>No concurrent provider/device calls were made. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T47" s="1"/>
     </x:row>
     <x:row r="48" ht="87" customHeight="1">
@@ -2773,9 +3009,15 @@
       <x:c r="P48" s="17" t="str">
         <x:v>2026-09-16: run-recovery.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q48" s="1"/>
-      <x:c r="R48" s="1"/>
-      <x:c r="S48" s="1"/>
+      <x:c r="Q48" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R48" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S48" s="17" t="str">
+        <x:v>Unknown-usage branch and model-mismatch case were not tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T48" s="1"/>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
@@ -2827,9 +3069,15 @@
       <x:c r="P49" s="19" t="str">
         <x:v>polished.js request errors; server.cjs; polished.js:193-255,380-422; intentgraph/server.cjs:206-285</x:v>
       </x:c>
-      <x:c r="Q49" s="1"/>
-      <x:c r="R49" s="1"/>
-      <x:c r="S49" s="1"/>
+      <x:c r="Q49" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R49" s="19" t="str">
+        <x:v>Current storage/API/browser replay uses the same receipt and never dispatches automatically. Partial: no live device or checkpoint resumption validation. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S49" s="19" t="str">
+        <x:v>No unsafe repeated device operation was reproduced. This is an implementation gap, not a confirmed execution defect. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T49" s="1"/>
     </x:row>
     <x:row r="50" ht="87" customHeight="1">
@@ -2881,9 +3129,15 @@
       <x:c r="P50" s="17" t="str">
         <x:v>2026-09-16: run-recovery.json; run-durability.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q50" s="1"/>
-      <x:c r="R50" s="1"/>
-      <x:c r="S50" s="1"/>
+      <x:c r="Q50" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R50" s="17" t="str">
+        <x:v>Current lost-response/reload and explicit owner-safe receipt recovery pass in WSL Chrome. Native Windows packaged restart remains unverified. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S50" s="17" t="str">
+        <x:v>This was an isolated browser/journal simulation, not a process crash of the packaged app. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T50" s="1"/>
     </x:row>
     <x:row r="51" ht="72" customHeight="1">
@@ -2935,9 +3189,15 @@
       <x:c r="P51" s="15" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/edit-rendering.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q51" s="1"/>
-      <x:c r="R51" s="1"/>
-      <x:c r="S51" s="1"/>
+      <x:c r="Q51" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R51" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S51" s="15" t="str">
+        <x:v>No substantive gap in the representative readability and inert-HTML slice; broader sanitizer fuzzing remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T51" s="1"/>
     </x:row>
     <x:row r="52" ht="117" customHeight="1">
@@ -2989,9 +3249,15 @@
       <x:c r="P52" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/runtime/verify-queue-terminal.cjs:77-118 (exact raw whitespace/copy); .intentgraph/evidence/ux-fixes-2026-09-15/root-review.json Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q52" s="1"/>
-      <x:c r="R52" s="1"/>
-      <x:c r="S52" s="1"/>
+      <x:c r="Q52" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R52" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S52" s="17" t="str">
+        <x:v>No substantive gap in the tested exact-copy and single-render slice; OS clipboard integration remains isolated. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T52" s="1"/>
     </x:row>
     <x:row r="53" ht="117" customHeight="1">
@@ -3043,9 +3309,15 @@
       <x:c r="P53" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (clipboard denial reports failure); .intentgraph/evidence/message-tools.json (answer/question copy) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q53" s="1"/>
-      <x:c r="R53" s="1"/>
-      <x:c r="S53" s="1"/>
+      <x:c r="Q53" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R53" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S53" s="19" t="str">
+        <x:v>No substantive gap in correct-copy and denied-clipboard feedback; OS clipboard integration remains isolated. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T53" s="1"/>
     </x:row>
     <x:row r="54" ht="87" customHeight="1">
@@ -3097,9 +3369,15 @@
       <x:c r="P54" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json; verify-history-navigation.cjs exit 0. Isolated mocked chat; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q54" s="1"/>
-      <x:c r="R54" s="1"/>
-      <x:c r="S54" s="1"/>
+      <x:c r="Q54" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R54" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S54" s="17" t="str">
+        <x:v>No substantive gap in old/new grouping and focused labels; timezone presentation matrix remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T54" s="1"/>
     </x:row>
     <x:row r="55" ht="87" customHeight="1">
@@ -3151,9 +3429,15 @@
       <x:c r="P55" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json; verify-history-navigation.cjs exit 0. Isolated mocked chat; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q55" s="1"/>
-      <x:c r="R55" s="1"/>
-      <x:c r="S55" s="1"/>
+      <x:c r="Q55" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R55" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S55" s="19" t="str">
+        <x:v>No substantive gap in the injected new-output/reading-position slice; live provider streaming is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T55" s="1"/>
     </x:row>
     <x:row r="56" ht="132" customHeight="1">
@@ -3205,9 +3489,15 @@
       <x:c r="P56" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-fixes-2026-09-15/history-regression.json (revert no execution, undo after reload); .intentgraph/runtime/verify-edit-rendering.cjs:1-16 (queued edit disabled) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q56" s="1"/>
-      <x:c r="R56" s="1"/>
-      <x:c r="S56" s="1"/>
+      <x:c r="Q56" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R56" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S56" s="17" t="str">
+        <x:v>The busy active-run protection branch is not exercised; queued-work protection alone does not close the full acceptance. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T56" s="1"/>
     </x:row>
     <x:row r="57" ht="87" customHeight="1">
@@ -3259,9 +3549,15 @@
       <x:c r="P57" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json; verify-history-navigation.cjs exit 0. Isolated mocked chat; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q57" s="1"/>
-      <x:c r="R57" s="1"/>
-      <x:c r="S57" s="1"/>
+      <x:c r="Q57" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R57" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S57" s="19" t="str">
+        <x:v>No substantive gap in fork provenance, parent immutability and reload revisit; cross-device sync remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T57" s="1"/>
     </x:row>
     <x:row r="58" ht="87" customHeight="1">
@@ -3313,9 +3609,15 @@
       <x:c r="P58" s="17" t="str">
         <x:v>2026-09-16: run-recovery.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q58" s="1"/>
-      <x:c r="R58" s="1"/>
-      <x:c r="S58" s="1"/>
+      <x:c r="Q58" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R58" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S58" s="17" t="str">
+        <x:v>No substantive gap in the v9 live existing/missing/archived local-link slice; external URL handling remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T58" s="1"/>
     </x:row>
     <x:row r="59" ht="117" customHeight="1">
@@ -3367,9 +3669,15 @@
       <x:c r="P59" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q59" s="1"/>
-      <x:c r="R59" s="1"/>
-      <x:c r="S59" s="1"/>
+      <x:c r="Q59" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R59" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S59" s="19" t="str">
+        <x:v>The reaction candidate covers search, contained keyboard navigation, Escape focus return and persistence, but its isolated candidate browser run is not a fresh served v9.1 run; screen-reader, visual-reference and multi-device checks remain outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T59" s="1"/>
     </x:row>
     <x:row r="60" ht="132" customHeight="1">
@@ -3421,9 +3729,15 @@
       <x:c r="P60" s="21" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/project-navigation.json (archive/restore/reload and busy guard); .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json (archived read-only) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q60" s="1"/>
-      <x:c r="R60" s="1"/>
-      <x:c r="S60" s="1"/>
+      <x:c r="Q60" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R60" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S60" s="21" t="str">
+        <x:v>The archive/restore check confirms composer state and one message, but does not deep-compare the full message/evidence payload before and after restore. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T60" s="1"/>
     </x:row>
     <x:row r="61" ht="117" customHeight="1">
@@ -3475,9 +3789,15 @@
       <x:c r="P61" s="19" t="str">
         <x:v>2026-09-15: local-data-ui.json; browser test exit 0. verify-backup-schema.cjs 9/9 passed, including private-field rejection, exact evidence, UTF-8 size boundary and interrupted-import recovery. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q61" s="1"/>
-      <x:c r="R61" s="1"/>
-      <x:c r="S61" s="1"/>
+      <x:c r="Q61" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R61" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S61" s="19" t="str">
+        <x:v>Export checks format, selected chat presence, pin metadata and token exclusion, but does not assert exact selected scope, timestamps and raw evidence comprehensively. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T61" s="1"/>
     </x:row>
     <x:row r="62" ht="117" customHeight="1">
@@ -3529,9 +3849,15 @@
       <x:c r="P62" s="17" t="str">
         <x:v>2026-09-15: local-data-ui.json; browser test exit 0. verify-backup-schema.cjs 9/9 passed, including private-field rejection, exact evidence, UTF-8 size boundary and interrupted-import recovery. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q62" s="1"/>
-      <x:c r="R62" s="1"/>
-      <x:c r="S62" s="1"/>
+      <x:c r="Q62" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R62" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S62" s="17" t="str">
+        <x:v>No substantive gap in invalid-JSON safety plus valid Add-mode preservation of unrelated work, pins and queues; the check is local-browser scoped. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T62" s="1"/>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
@@ -3583,9 +3909,15 @@
       <x:c r="P63" s="19" t="str">
         <x:v>architecture.json; polished.js persistence; polished.js:19-58,158-174,460,481</x:v>
       </x:c>
-      <x:c r="Q63" s="1"/>
-      <x:c r="R63" s="1"/>
-      <x:c r="S63" s="1"/>
+      <x:c r="Q63" s="19" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="R63" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S63" s="19" t="str">
+        <x:v>No cross-device service exists in this build. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T63" s="1"/>
     </x:row>
     <x:row r="64" ht="132" customHeight="1">
@@ -3637,9 +3969,15 @@
       <x:c r="P64" s="21" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/avatar-family-app-qa-results.json (all avatar choices/custom color/photo/migration/reload; no external requests); .intentgraph/runtime/verify-backup-schema.cjs:4,15-28 Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q64" s="1"/>
-      <x:c r="R64" s="1"/>
-      <x:c r="S64" s="1"/>
+      <x:c r="Q64" s="21" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R64" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S64" s="21" t="str">
+        <x:v>No substantive gap in legacy avatar normalization, chosen avatar persistence and reload; the check uses one legacy fixture. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T64" s="1"/>
     </x:row>
     <x:row r="65" ht="132" customHeight="1">
@@ -3691,9 +4029,15 @@
       <x:c r="P65" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-fixes-2026-09-15/root-identity-review.json (profile identity/rename sync); .intentgraph/avatar-family-app-qa-results.json (long-name responsive fixture) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q65" s="1"/>
-      <x:c r="R65" s="1"/>
-      <x:c r="S65" s="1"/>
+      <x:c r="Q65" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R65" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S65" s="19" t="str">
+        <x:v>The long label remains selected-only, but only one long name is exercised and persisted reload of the saved edit is not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T65" s="1"/>
     </x:row>
     <x:row r="66" ht="87" customHeight="1">
@@ -3745,9 +4089,15 @@
       <x:c r="P66" s="17" t="str">
         <x:v>2026-09-16: pane-controls.json. Remaining scope is explicit; not marked complete.</x:v>
       </x:c>
-      <x:c r="Q66" s="1"/>
-      <x:c r="R66" s="1"/>
-      <x:c r="S66" s="1"/>
+      <x:c r="Q66" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R66" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S66" s="17" t="str">
+        <x:v>Saving and consuming the same document in a real model request were not demonstrated. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T66" s="1"/>
     </x:row>
     <x:row r="67" ht="72" customHeight="1">
@@ -3799,9 +4149,15 @@
       <x:c r="P67" s="19" t="str">
         <x:v>2026-09-16: alerts.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q67" s="1"/>
-      <x:c r="R67" s="1"/>
-      <x:c r="S67" s="1"/>
+      <x:c r="Q67" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R67" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S67" s="19" t="str">
+        <x:v>Finished enabled and muted paths pass, but waiting/error alert variants remain owned by the unintegrated automation alert core. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T67" s="1"/>
     </x:row>
     <x:row r="68" ht="70" customHeight="1">
@@ -3853,9 +4209,15 @@
       <x:c r="P68" s="17" t="str">
         <x:v>2026-09-16: accessibility-results.json UX058. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q68" s="1"/>
-      <x:c r="R68" s="1"/>
-      <x:c r="S68" s="1"/>
+      <x:c r="Q68" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R68" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S68" s="17" t="str">
+        <x:v>No substantive gap in local welcome semantics and persisted first-chat behavior; no model/provider request or cross-device storage is exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T68" s="1"/>
     </x:row>
     <x:row r="69" ht="117" customHeight="1">
@@ -3907,9 +4269,15 @@
       <x:c r="P69" s="15" t="str">
         <x:v>2026-09-15: local-data-ui.json; browser test exit 0. verify-backup-schema.cjs 9/9 passed, including private-field rejection, exact evidence, UTF-8 size boundary and interrupted-import recovery. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q69" s="1"/>
-      <x:c r="R69" s="1"/>
-      <x:c r="S69" s="1"/>
+      <x:c r="Q69" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R69" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S69" s="15" t="str">
+        <x:v>Both theme colors/readability and save/cancel pass, but persistence across a reload is not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T69" s="1"/>
     </x:row>
     <x:row r="70" ht="87" customHeight="1">
@@ -3961,9 +4329,15 @@
       <x:c r="P70" s="17" t="str">
         <x:v>2026-09-16: diagnostics-ui.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q70" s="1"/>
-      <x:c r="R70" s="1"/>
-      <x:c r="S70" s="1"/>
+      <x:c r="Q70" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R70" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S70" s="17" t="str">
+        <x:v>Local configured status is not proof of provider reachability; no credentials or provider requests were used. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T70" s="1"/>
     </x:row>
     <x:row r="71" ht="72" customHeight="1">
@@ -4015,9 +4389,15 @@
       <x:c r="P71" s="19" t="str">
         <x:v>2026-09-16: diagnostics-ui.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q71" s="1"/>
-      <x:c r="R71" s="1"/>
-      <x:c r="S71" s="1"/>
+      <x:c r="Q71" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R71" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S71" s="19" t="str">
+        <x:v>No remote adapter health check or inventory load was performed. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T71" s="1"/>
     </x:row>
     <x:row r="72" ht="102" customHeight="1">
@@ -4069,9 +4449,15 @@
       <x:c r="P72" s="17" t="str">
         <x:v>2026-09-16: verify-local-data-ui.cjs; verify-backup-schema.cjs 10 tests; attachments.json. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q72" s="1"/>
-      <x:c r="R72" s="1"/>
-      <x:c r="S72" s="1"/>
+      <x:c r="Q72" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R72" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S72" s="17" t="str">
+        <x:v>The privacy wording passes, while destructive reset/recovery behavior is not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T72" s="1"/>
     </x:row>
     <x:row r="73" ht="42" customHeight="1">
@@ -4123,9 +4509,15 @@
       <x:c r="P73" s="19" t="str">
         <x:v>A0; polished.html account-menu; polished.js:480-482</x:v>
       </x:c>
-      <x:c r="Q73" s="1"/>
-      <x:c r="R73" s="1"/>
-      <x:c r="S73" s="1"/>
+      <x:c r="Q73" s="19" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="R73" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S73" s="19" t="str">
+        <x:v>No remote identity is connected. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T73" s="1"/>
     </x:row>
     <x:row r="74" ht="87" customHeight="1">
@@ -4177,9 +4569,15 @@
       <x:c r="P74" s="17" t="str">
         <x:v>2026-09-16: diagnostics-ui.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q74" s="1"/>
-      <x:c r="R74" s="1"/>
-      <x:c r="S74" s="1"/>
+      <x:c r="Q74" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R74" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S74" s="17" t="str">
+        <x:v>Only one help entry and a successful local feedback save are checked; every-help coverage and feedback storage failure are absent. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T74" s="1"/>
     </x:row>
     <x:row r="75" ht="72" customHeight="1">
@@ -4231,9 +4629,15 @@
       <x:c r="P75" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/local-commands.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q75" s="1"/>
-      <x:c r="R75" s="1"/>
-      <x:c r="S75" s="1"/>
+      <x:c r="Q75" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R75" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S75" s="19" t="str">
+        <x:v>Ctrl+K and displayed shortcut text pass, but Cmd/Ctrl+F behavior and unavailable-action filtering are not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T75" s="1"/>
     </x:row>
     <x:row r="76" ht="87" customHeight="1">
@@ -4285,9 +4689,15 @@
       <x:c r="P76" s="21" t="str">
         <x:v>2026-09-16: workspace-shell.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q76" s="1"/>
-      <x:c r="R76" s="1"/>
-      <x:c r="S76" s="1"/>
+      <x:c r="Q76" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R76" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S76" s="21" t="str">
+        <x:v>Deduplication fix verified for unambiguous mirrored results; broader artifact-file capability remains partial. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T76" s="1"/>
     </x:row>
     <x:row r="77" ht="72" customHeight="1">
@@ -4339,9 +4749,15 @@
       <x:c r="P77" s="19" t="str">
         <x:v>2026-09-16: pane-controls.json. Remaining scope is explicit; not marked complete.</x:v>
       </x:c>
-      <x:c r="Q77" s="1"/>
-      <x:c r="R77" s="1"/>
-      <x:c r="S77" s="1"/>
+      <x:c r="Q77" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R77" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S77" s="19" t="str">
+        <x:v>Unavailable state passed; live browsing capability remains absent. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T77" s="1"/>
     </x:row>
     <x:row r="78" ht="87" customHeight="1">
@@ -4393,9 +4809,15 @@
       <x:c r="P78" s="17" t="str">
         <x:v>2026-09-16: pane-controls.json. Remaining scope is explicit; not marked complete.</x:v>
       </x:c>
-      <x:c r="Q78" s="1"/>
-      <x:c r="R78" s="1"/>
-      <x:c r="S78" s="1"/>
+      <x:c r="Q78" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R78" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S78" s="17" t="str">
+        <x:v>Unavailable state passed; live computer control remains absent. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T78" s="1"/>
     </x:row>
     <x:row r="79" ht="87" customHeight="1">
@@ -4447,9 +4869,15 @@
       <x:c r="P79" s="19" t="str">
         <x:v>2026-09-16: pane-controls.json. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q79" s="1"/>
-      <x:c r="R79" s="1"/>
-      <x:c r="S79" s="1"/>
+      <x:c r="Q79" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R79" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S79" s="19" t="str">
+        <x:v>One keyboard resize and focus return pass, but evidence-specific read/type room and a broader resize matrix are not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T79" s="1"/>
     </x:row>
     <x:row r="80" ht="102" customHeight="1">
@@ -4501,9 +4929,15 @@
       <x:c r="P80" s="17" t="str">
         <x:v>2026-09-16: verify-local-files.cjs 34 checks; files-shell.json 26 checks with real Web Crypto and memory-only file handles. No user disk writes. Real OS picker and owner acceptance remain unverified.</x:v>
       </x:c>
-      <x:c r="Q80" s="1"/>
-      <x:c r="R80" s="1"/>
-      <x:c r="S80" s="1"/>
+      <x:c r="Q80" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R80" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S80" s="17" t="str">
+        <x:v>No user disk writes were performed. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T80" s="1"/>
     </x:row>
     <x:row r="81" ht="42" customHeight="1">
@@ -4555,9 +4989,15 @@
       <x:c r="P81" s="19" t="str">
         <x:v>architecture.json; polished.js; polished.js:319-370</x:v>
       </x:c>
-      <x:c r="Q81" s="1"/>
-      <x:c r="R81" s="1"/>
-      <x:c r="S81" s="1"/>
+      <x:c r="Q81" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R81" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S81" s="19" t="str">
+        <x:v>Intentional scope gap. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T81" s="1"/>
     </x:row>
     <x:row r="82" ht="102" customHeight="1">
@@ -4609,9 +5049,15 @@
       <x:c r="P82" s="21" t="str">
         <x:v>2026-09-16: files-shell.json passed. Verified local file slice only; network configuration review is not claimed.</x:v>
       </x:c>
-      <x:c r="Q82" s="1"/>
-      <x:c r="R82" s="1"/>
-      <x:c r="S82" s="1"/>
+      <x:c r="Q82" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R82" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S82" s="21" t="str">
+        <x:v>No network configuration calls were made. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T82" s="1"/>
     </x:row>
     <x:row r="83" ht="87" customHeight="1">
@@ -4663,9 +5109,15 @@
       <x:c r="P83" s="19" t="str">
         <x:v>2026-09-16: evidence-shell/evidence-shell-results.json 11 checks. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q83" s="1"/>
-      <x:c r="R83" s="1"/>
-      <x:c r="S83" s="1"/>
+      <x:c r="Q83" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R83" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S83" s="19" t="str">
+        <x:v>A successful annotation is saved, but stale-result rejection, discard and save-failure paths are not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T83" s="1"/>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
@@ -4717,9 +5169,15 @@
       <x:c r="P84" s="17" t="str">
         <x:v>intentgraph/adapters/index.cjs:462-503,570-598; polished.js:359-370</x:v>
       </x:c>
-      <x:c r="Q84" s="1"/>
-      <x:c r="R84" s="1"/>
-      <x:c r="S84" s="1"/>
+      <x:c r="Q84" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R84" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S84" s="17" t="str">
+        <x:v>No execution or provider calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T84" s="1"/>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
@@ -4771,9 +5229,15 @@
       <x:c r="P85" s="19" t="str">
         <x:v>polished.html; polished.js; intentgraph/adapters/index.cjs:462-503,570-598; polished.js:359-370</x:v>
       </x:c>
-      <x:c r="Q85" s="1"/>
-      <x:c r="R85" s="1"/>
-      <x:c r="S85" s="1"/>
+      <x:c r="Q85" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R85" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S85" s="19" t="str">
+        <x:v>No Git operation was attempted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T85" s="1"/>
     </x:row>
     <x:row r="86" ht="42" customHeight="1">
@@ -4825,9 +5289,15 @@
       <x:c r="P86" s="21" t="str">
         <x:v>polished.js:332-357; intentgraph/agent-runtime.cjs:271-338</x:v>
       </x:c>
-      <x:c r="Q86" s="1"/>
-      <x:c r="R86" s="1"/>
-      <x:c r="S86" s="1"/>
+      <x:c r="Q86" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R86" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S86" s="21" t="str">
+        <x:v>Inventory route was mocked and no device call was made. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T86" s="1"/>
     </x:row>
     <x:row r="87" ht="72" customHeight="1">
@@ -4879,9 +5349,15 @@
       <x:c r="P87" s="19" t="str">
         <x:v>2026-09-16: pane-controls.json; verify-chat-modes.cjs. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q87" s="1"/>
-      <x:c r="R87" s="1"/>
-      <x:c r="S87" s="1"/>
+      <x:c r="Q87" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R87" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S87" s="19" t="str">
+        <x:v>No live device call or enforcement backend was used. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T87" s="1"/>
     </x:row>
     <x:row r="88" ht="132" customHeight="1">
@@ -4933,9 +5409,15 @@
       <x:c r="P88" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (Markdown has run-42 and command/target); .intentgraph/evidence/ux-fixes-2026-09-15/local-data-ui.json (raw export) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q88" s="1"/>
-      <x:c r="R88" s="1"/>
-      <x:c r="S88" s="1"/>
+      <x:c r="Q88" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R88" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S88" s="17" t="str">
+        <x:v>Exact copied/exported evidence provenance across all timestamps and commands was not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T88" s="1"/>
     </x:row>
     <x:row r="89" ht="102" customHeight="1">
@@ -4987,9 +5469,15 @@
       <x:c r="P89" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. preserved-audit.json: top-level SUCCESS with nested FAILURE renders FAILURE; run state outcome precedence verified Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q89" s="1"/>
-      <x:c r="R89" s="1"/>
-      <x:c r="S89" s="1"/>
+      <x:c r="Q89" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R89" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S89" s="19" t="str">
+        <x:v>The device health conclusion is fixture-driven. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T89" s="1"/>
     </x:row>
     <x:row r="90" ht="42" customHeight="1">
@@ -5041,9 +5529,15 @@
       <x:c r="P90" s="17" t="str">
         <x:v>architecture.json; intentgraph/agent-runtime.cjs:203-214,271-415</x:v>
       </x:c>
-      <x:c r="Q90" s="1"/>
-      <x:c r="R90" s="1"/>
-      <x:c r="S90" s="1"/>
+      <x:c r="Q90" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R90" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S90" s="17" t="str">
+        <x:v>No state-changing workflow is present to exercise. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T90" s="1"/>
     </x:row>
     <x:row r="91" ht="87" customHeight="1">
@@ -5095,9 +5589,15 @@
       <x:c r="P91" s="19" t="str">
         <x:v>2026-09-16: evidence-shell/evidence-shell-results.json; verify-evidence-tools.cjs. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q91" s="1"/>
-      <x:c r="R91" s="1"/>
-      <x:c r="S91" s="1"/>
+      <x:c r="Q91" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R91" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S91" s="19" t="str">
+        <x:v>The comparison UI and timestamp labeling across different runs were not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T91" s="1"/>
     </x:row>
     <x:row r="92" ht="42" customHeight="1">
@@ -5149,9 +5649,15 @@
       <x:c r="P92" s="17" t="str">
         <x:v>Runtime/output verification needed; intentgraph/agent-runtime.cjs:203-214,271-415</x:v>
       </x:c>
-      <x:c r="Q92" s="1"/>
-      <x:c r="R92" s="1"/>
-      <x:c r="S92" s="1"/>
+      <x:c r="Q92" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R92" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S92" s="17" t="str">
+        <x:v>No topology data contract or renderer in Aven shell. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T92" s="1"/>
     </x:row>
     <x:row r="93" ht="87" customHeight="1">
@@ -5203,9 +5709,15 @@
       <x:c r="P93" s="15" t="str">
         <x:v>2026-09-16: workspace-shell.json; verify-workspace-tools.cjs 30 checks. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q93" s="1"/>
-      <x:c r="R93" s="1"/>
-      <x:c r="S93" s="1"/>
+      <x:c r="Q93" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R93" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S93" s="15" t="str">
+        <x:v>Only the empty Feed explanation is exercised; populated entries opening their distinct saved runs are not. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T93" s="1"/>
     </x:row>
     <x:row r="94" ht="87" customHeight="1">
@@ -5257,9 +5769,15 @@
       <x:c r="P94" s="17" t="str">
         <x:v>2026-09-16: workspace-shell.json; verify-workspace-tools.cjs 30 checks. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q94" s="1"/>
-      <x:c r="R94" s="1"/>
-      <x:c r="S94" s="1"/>
+      <x:c r="Q94" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R94" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S94" s="17" t="str">
+        <x:v>No substantive gap in local idea add/save/reload/archive/restore behavior; no remote persistence is exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T94" s="1"/>
     </x:row>
     <x:row r="95" ht="87" customHeight="1">
@@ -5311,9 +5829,15 @@
       <x:c r="P95" s="19" t="str">
         <x:v>2026-09-16: verify-workspace-tools.cjs 30 checks; workspace-shell.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q95" s="1"/>
-      <x:c r="R95" s="1"/>
-      <x:c r="S95" s="1"/>
+      <x:c r="Q95" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R95" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S95" s="19" t="str">
+        <x:v>The child module check only inspected source text. Completion, persistence and invalid-evidence rejection were not behaviorally tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T95" s="1"/>
     </x:row>
     <x:row r="96" ht="42" customHeight="1">
@@ -5365,9 +5889,15 @@
       <x:c r="P96" s="17" t="str">
         <x:v>polished.html; server.cjs; polished.js:434-449; intentgraph/ui/index.html:7-8</x:v>
       </x:c>
-      <x:c r="Q96" s="1"/>
-      <x:c r="R96" s="1"/>
-      <x:c r="S96" s="1"/>
+      <x:c r="Q96" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R96" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S96" s="17" t="str">
+        <x:v>No scheduler surface exists. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T96" s="1"/>
     </x:row>
     <x:row r="97" ht="72" customHeight="1">
@@ -5419,9 +5949,15 @@
       <x:c r="P97" s="19" t="str">
         <x:v>2026-09-16: alerts.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q97" s="1"/>
-      <x:c r="R97" s="1"/>
-      <x:c r="S97" s="1"/>
+      <x:c r="Q97" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R97" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S97" s="19" t="str">
+        <x:v>The enabled preference and finished-result path are covered through UX-057, but waiting/error variants and duplicate visible-alert suppression are not. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T97" s="1"/>
     </x:row>
     <x:row r="98" ht="42" customHeight="1">
@@ -5473,9 +6009,15 @@
       <x:c r="P98" s="17" t="str">
         <x:v>polished.html plugins pane; polished.js:434-449; intentgraph/ui/index.html:7-8</x:v>
       </x:c>
-      <x:c r="Q98" s="1"/>
-      <x:c r="R98" s="1"/>
-      <x:c r="S98" s="1"/>
+      <x:c r="Q98" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R98" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S98" s="17" t="str">
+        <x:v>Local fixtures only; no provider/device calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T98" s="1"/>
     </x:row>
     <x:row r="99" ht="42" customHeight="1">
@@ -5527,9 +6069,15 @@
       <x:c r="P99" s="19" t="str">
         <x:v>polished.js documents; runtime; polished.js:434-449; intentgraph/ui/index.html:7-8</x:v>
       </x:c>
-      <x:c r="Q99" s="1"/>
-      <x:c r="R99" s="1"/>
-      <x:c r="S99" s="1"/>
+      <x:c r="Q99" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R99" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S99" s="19" t="str">
+        <x:v>Local documents exist, but the requested reusable workflow capability is absent. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T99" s="1"/>
     </x:row>
     <x:row r="100" ht="42" customHeight="1">
@@ -5581,9 +6129,15 @@
       <x:c r="P100" s="17" t="str">
         <x:v>architecture.json; polished.js:434-449; intentgraph/ui/index.html:7-8</x:v>
       </x:c>
-      <x:c r="Q100" s="1"/>
-      <x:c r="R100" s="1"/>
-      <x:c r="S100" s="1"/>
+      <x:c r="Q100" s="17" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="R100" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S100" s="17" t="str">
+        <x:v>Deferred by user decision. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T100" s="1"/>
     </x:row>
     <x:row r="101" ht="72" customHeight="1">
@@ -5635,9 +6189,15 @@
       <x:c r="P101" s="15" t="str">
         <x:v>2026-09-16: accessibility-results.json; pane-controls.json. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q101" s="1"/>
-      <x:c r="R101" s="1"/>
-      <x:c r="S101" s="1"/>
+      <x:c r="Q101" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R101" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S101" s="15" t="str">
+        <x:v>Plus/settings keyboard paths pass, but all visible controls, full logical order, trap detection and every Escape return are not covered. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T101" s="1"/>
     </x:row>
     <x:row r="102" ht="72" customHeight="1">
@@ -5689,9 +6249,15 @@
       <x:c r="P102" s="17" t="str">
         <x:v>2026-09-16: accessibility-results.json UX092; no full WCAG conformance claim. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q102" s="1"/>
-      <x:c r="R102" s="1"/>
-      <x:c r="S102" s="1"/>
+      <x:c r="Q102" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R102" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S102" s="17" t="str">
+        <x:v>Representative ARIA roles/names and selected state pass, but there is no screen-reader run covering every action, coworker and active-run state. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T102" s="1"/>
     </x:row>
     <x:row r="103" ht="87" customHeight="1">
@@ -5743,9 +6309,15 @@
       <x:c r="P103" s="19" t="str">
         <x:v>2026-09-16: accessibility-results.json; scoped checks, not a full WCAG conformance claim. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q103" s="1"/>
-      <x:c r="R103" s="1"/>
-      <x:c r="S103" s="1"/>
+      <x:c r="Q103" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R103" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S103" s="19" t="str">
+        <x:v>One answer contrast measurement and 200% narrow overflow check pass, but all controls and a broader narrow/reflow matrix are not measured. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T103" s="1"/>
     </x:row>
     <x:row r="104" ht="72" customHeight="1">
@@ -5797,9 +6369,15 @@
       <x:c r="P104" s="17" t="str">
         <x:v>2026-09-16: accessibility-results.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q104" s="1"/>
-      <x:c r="R104" s="1"/>
-      <x:c r="S104" s="1"/>
+      <x:c r="Q104" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R104" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S104" s="17" t="str">
+        <x:v>Decorative animation is disabled under reduced motion, but state-changing interactions under the preference are not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T104" s="1"/>
     </x:row>
     <x:row r="105" ht="72" customHeight="1">
@@ -5851,9 +6429,15 @@
       <x:c r="P105" s="19" t="str">
         <x:v>2026-09-16: accessibility-results.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q105" s="1"/>
-      <x:c r="R105" s="1"/>
-      <x:c r="S105" s="1"/>
+      <x:c r="Q105" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R105" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S105" s="19" t="str">
+        <x:v>Touch target sizes pass, but hover menu bounds, close behavior and focus restoration are not covered by this quality check. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T105" s="1"/>
     </x:row>
     <x:row r="106" ht="72" customHeight="1">
@@ -5905,9 +6489,15 @@
       <x:c r="P106" s="17" t="str">
         <x:v>2026-09-16: accessibility-results.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q106" s="1"/>
-      <x:c r="R106" s="1"/>
-      <x:c r="S106" s="1"/>
+      <x:c r="Q106" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R106" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S106" s="17" t="str">
+        <x:v>A 320px pane open/close and containment check passes, but desktop/zoomed controls and deliberate table scrolling are not covered. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T106" s="1"/>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
@@ -5959,9 +6549,15 @@
       <x:c r="P107" s="19" t="str">
         <x:v>A0 Feed, Artifacts, Settings; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q107" s="1"/>
-      <x:c r="R107" s="1"/>
-      <x:c r="S107" s="1"/>
+      <x:c r="Q107" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R107" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S107" s="19" t="str">
+        <x:v>Unavailable context is truthful, but the evidence does not enumerate every visible action and its real result/unavailable explanation. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T107" s="1"/>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
@@ -6013,9 +6609,15 @@
       <x:c r="P108" s="17" t="str">
         <x:v>polished.js request handlers; server.cjs; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q108" s="1"/>
-      <x:c r="R108" s="1"/>
-      <x:c r="S108" s="1"/>
+      <x:c r="Q108" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R108" s="17" t="str">
+        <x:v>Current local storage, response-loss, cancellation and persistence-failure fixtures preserve draft/evidence and explicit review. Provider-specific errors remain mocked; no live reachability proof. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S108" s="17" t="str">
+        <x:v>Only the creation transaction/reload/retry path was fixed and tested in this batch. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T108" s="1"/>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
@@ -6067,9 +6669,15 @@
       <x:c r="P109" s="19" t="str">
         <x:v>Performance check not run; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q109" s="1"/>
-      <x:c r="R109" s="1"/>
-      <x:c r="S109" s="1"/>
+      <x:c r="Q109" s="19" t="str">
+        <x:v>Unverified</x:v>
+      </x:c>
+      <x:c r="R109" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S109" s="19" t="str">
+        <x:v>A browser-control timeout occurred on the live artifact view; cause was not isolated and is not counted as a product defect. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T109" s="1"/>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
@@ -6121,9 +6729,15 @@
       <x:c r="P110" s="17" t="str">
         <x:v>A0; polished.js initialization; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q110" s="1"/>
-      <x:c r="R110" s="1"/>
-      <x:c r="S110" s="1"/>
+      <x:c r="Q110" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R110" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S110" s="17" t="str">
+        <x:v>Provider/device readiness and selected device are not part of onboarding. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T110" s="1"/>
     </x:row>
     <x:row r="111" ht="177" customHeight="1">
@@ -6175,9 +6789,15 @@
       <x:c r="P111" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/runtime/verify-backup-schema.cjs:4-28 (current six backup/transaction/size tests); .intentgraph/evidence/ux-fixes-2026-09-15/local-data-ui.json (roundtrip/Add/replace/reload); .intentgraph/evidence/ux-fixes-2026-09-15/history-regression.json (revert/avatar/history) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q111" s="1"/>
-      <x:c r="R111" s="1"/>
-      <x:c r="S111" s="1"/>
+      <x:c r="Q111" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R111" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S111" s="19" t="str">
+        <x:v>It did not prove exact migration preservation of all chats, drafts, queues, avatars and revert history. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T111" s="1"/>
     </x:row>
     <x:row r="112" ht="87" customHeight="1">
@@ -6229,9 +6849,15 @@
       <x:c r="P112" s="17" t="str">
         <x:v>2026-09-16: diagnostics-ui.json; verify-chat-read-api.cjs. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q112" s="1"/>
-      <x:c r="R112" s="1"/>
-      <x:c r="S112" s="1"/>
+      <x:c r="Q112" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R112" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S112" s="17" t="str">
+        <x:v>Local status fixtures and served build identity only; no live provider/device reachability claim. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T112" s="1"/>
     </x:row>
     <x:row r="113" ht="117" customHeight="1">
@@ -6283,9 +6909,15 @@
       <x:c r="P113" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q113" s="1"/>
-      <x:c r="R113" s="1"/>
-      <x:c r="S113" s="1"/>
+      <x:c r="Q113" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R113" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S113" s="19" t="str">
+        <x:v>The known rename inconsistency is resolved; complete terminology and icon acceptance is not yet verified. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T113" s="1"/>
     </x:row>
     <x:row r="114" ht="42" customHeight="1">
@@ -6337,9 +6969,15 @@
       <x:c r="P114" s="17" t="str">
         <x:v>architecture.json; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q114" s="1"/>
-      <x:c r="R114" s="1"/>
-      <x:c r="S114" s="1"/>
+      <x:c r="Q114" s="17" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="R114" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S114" s="17" t="str">
+        <x:v>Deferred by user decision. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T114" s="1"/>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
@@ -6391,9 +7029,15 @@
       <x:c r="P115" s="19" t="str">
         <x:v>User feedback; current audit; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q115" s="1"/>
-      <x:c r="R115" s="1"/>
-      <x:c r="S115" s="1"/>
+      <x:c r="Q115" s="19" t="str">
+        <x:v>Unverified</x:v>
+      </x:c>
+      <x:c r="R115" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S115" s="19" t="str">
+        <x:v>Owner acceptance unavailable. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T115" s="1"/>
     </x:row>
     <x:row r="116" ht="132" customHeight="1">
@@ -6445,9 +7089,15 @@
       <x:c r="P116" s="21" t="str">
         <x:v>2026-09-16: preservation audit PASS. 25/25 local fixture tests passed: agent-runtime/chat-runtime/network-execution/sandbox-routes/steering suites (allowlist, exact target, failed transport, read-only origin/header); no provider/device calls Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q116" s="1"/>
-      <x:c r="R116" s="1"/>
-      <x:c r="S116" s="1"/>
+      <x:c r="Q116" s="21" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R116" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S116" s="21" t="str">
+        <x:v>Local fixtures only; no provider/device calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T116" s="1"/>
     </x:row>
     <x:row r="117" ht="87" customHeight="1">
@@ -6499,9 +7149,15 @@
       <x:c r="P117" s="19" t="str">
         <x:v>2026-09-16: verify-queue-terminal.cjs 4/4; run-durability.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q117" s="1"/>
-      <x:c r="R117" s="1"/>
-      <x:c r="S117" s="1"/>
+      <x:c r="Q117" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R117" s="19" t="str">
+        <x:v>Cancellation and dead-owner recovery remain UNKNOWN; replay and recovery cause no duplicate fixture responder invocation. No claim of stopping a remote device command. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S117" s="19" t="str">
+        <x:v>Stop UX and duplicate-retry prevention were not freshly exercised; no provider/device calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T117" s="1"/>
     </x:row>
     <x:row r="118" ht="87" customHeight="1">
@@ -6553,9 +7209,15 @@
       <x:c r="P118" s="21" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/chat-interactions.json; verify-chat-interactions.cjs exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q118" s="1"/>
-      <x:c r="R118" s="1"/>
-      <x:c r="S118" s="1"/>
+      <x:c r="Q118" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R118" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S118" s="21" t="str">
+        <x:v>A fresh over-limit request/omission-count comparison was not completed. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T118" s="1"/>
     </x:row>
     <x:row r="119" ht="117" customHeight="1">
@@ -6607,9 +7269,15 @@
       <x:c r="P119" s="15" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q119" s="1"/>
-      <x:c r="R119" s="1"/>
-      <x:c r="S119" s="1"/>
+      <x:c r="Q119" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R119" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S119" s="15" t="str">
+        <x:v>This audit did not save a note and inspect the next model request to verify exclusion. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T119" s="1"/>
     </x:row>
     <x:row r="120" ht="87" customHeight="1">
@@ -6661,9 +7329,15 @@
       <x:c r="P120" s="21" t="str">
         <x:v>2026-09-15: edit-rendering.json and verify-edit-rendering.cjs exit 0 validate safe-link slice only. Full media acceptance remains pending.</x:v>
       </x:c>
-      <x:c r="Q120" s="1"/>
-      <x:c r="R120" s="1"/>
-      <x:c r="S120" s="1"/>
+      <x:c r="Q120" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R120" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S120" s="21" t="str">
+        <x:v>Inline media and attachment reading remain pending. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T120" s="1"/>
     </x:row>
     <x:row r="121" ht="102" customHeight="1">
@@ -6715,9 +7389,15 @@
       <x:c r="P121" s="15" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (beforeOpen=true, afterOpen=false; no request path) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q121" s="1"/>
-      <x:c r="R121" s="1"/>
-      <x:c r="S121" s="1"/>
+      <x:c r="Q121" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R121" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S121" s="15" t="str">
+        <x:v>All exercised browser-local unread/reload/open and held local-run switching checks pass; provider execution and assistive-technology coverage remain outside this review. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T121" s="1"/>
     </x:row>
     <x:row r="122" ht="72" customHeight="1">
@@ -6769,9 +7449,15 @@
       <x:c r="P122" s="21" t="str">
         <x:v>2026-09-16: diagnostics-ui.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q122" s="1"/>
-      <x:c r="R122" s="1"/>
-      <x:c r="S122" s="1"/>
+      <x:c r="Q122" s="21" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R122" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S122" s="21" t="str">
+        <x:v>English fallback and disabled unsupported-language disclosure pass; additional translation coverage remains outside this review. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T122" s="1"/>
     </x:row>
     <x:row r="123" ht="87" customHeight="1">
@@ -6823,9 +7509,15 @@
       <x:c r="P123" s="15" t="str">
         <x:v>2026-09-16: alerts.json; verify-queue-terminal.cjs 4/4. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q123" s="1"/>
-      <x:c r="R123" s="1"/>
-      <x:c r="S123" s="1"/>
+      <x:c r="Q123" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R123" s="15" t="str">
+        <x:v>Active API enforces serial capacity; current browser waiting/draft fixture and queue checks supplement prior evidence. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S123" s="15" t="str">
+        <x:v>Full serial multi-conversation queue UI was not exercised in this bounded run. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T123" s="1"/>
     </x:row>
     <x:row r="124" ht="42" customHeight="1">
@@ -6877,9 +7569,15 @@
       <x:c r="P124" s="21" t="str">
         <x:v>intentgraph/ui/index.html:7-8; adapters/index.cjs:462-503,570-598</x:v>
       </x:c>
-      <x:c r="Q124" s="1"/>
-      <x:c r="R124" s="1"/>
-      <x:c r="S124" s="1"/>
+      <x:c r="Q124" s="21" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R124" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S124" s="21" t="str">
+        <x:v>Local fixtures only; no provider/device calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T124" s="1"/>
     </x:row>
     <x:row r="125" ht="132" customHeight="1">
@@ -6931,9 +7629,15 @@
       <x:c r="P125" s="15" t="str">
         <x:v>2026-09-16: preservation audit PASS. isolated `verify-chat-read-api.cjs` passed (original raw provenance/read-back; secret fields stripped); .intentgraph/evidence/pending-88-20260916/run-recovery.json (reload/deep links/durable capture) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q125" s="1"/>
-      <x:c r="R125" s="1"/>
-      <x:c r="S125" s="1"/>
+      <x:c r="Q125" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R125" s="15" t="str">
+        <x:v>Current scoped receipt and raw-run readback preserve original run/request/chat provenance and exact output. Evidence and admission settlement are distinct. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S125" s="15" t="str">
+        <x:v>Existing local records only; no new provider/device run, service restart or cross-device durability test. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T125" s="1"/>
     </x:row>
     <x:row r="126">
@@ -7767,7 +8471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b91acc2d02d4683"/>
+    <x:tablePart r:id="R3b91acc2d02d4683"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile pending chats independently and retain retry result identity
</commit_message>
<xml_diff>
--- a/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
+++ b/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
@@ -407,7 +407,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF253448"/>
   </x:sheetPr>
@@ -658,7 +658,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="str">
-        <x:v>19 September 2026: Q–S contain effective scoped verdicts and admission evidence. A–P and the summary above remain dated history. Counts: 37 scoped Verified, 57 Partial, 3 Unverified, 14 Missing, 4 Deferred; owner approval is separate.</x:v>
+        <x:v>19 September 2026: Q–S contain effective scoped verdicts and admission evidence. A–P and the summary above remain dated history. Counts: 37 scoped Verified, 57 Partial, 3 Unverified, 14 Missing, 4 Deferred; owner approval is separate. Independent-review recovery corrections are appended in R; verdict counts are unchanged.</x:v>
       </x:c>
       <x:c r="B9" s="1"/>
       <x:c r="C9" s="1"/>
@@ -2533,7 +2533,8 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="R40" s="17" t="str">
-        <x:v>Stable saved identities and backend duplicate suppression; current browser FIFO and explicit paused-queue checks. Broader crash-at-every-queue-boundary coverage remains partial. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+        <x:v>Stable saved identities and backend duplicate suppression; current browser FIFO and explicit paused-queue checks. Broader crash-at-every-queue-boundary coverage remains partial. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Mounted three-turn FIFO dispatches once per identity after writer-lock release; paused queues survive independent pending-chat recovery. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
       </x:c>
       <x:c r="S40" s="17" t="str">
         <x:v>Order and duplicate-submission behavior were not freshly exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
@@ -3073,7 +3074,8 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="R49" s="19" t="str">
-        <x:v>Current storage/API/browser replay uses the same receipt and never dispatches automatically. Partial: no live device or checkpoint resumption validation. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+        <x:v>Current storage/API/browser replay uses the same receipt and never dispatches automatically. Partial: no live device or checkpoint resumption validation. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Outage -&gt; missing receipt -&gt; successful Retry saved request updates one original message and retains timestamp, annotations and raw capture; no contradictory UNKNOWN/SUCCESS pair. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
       </x:c>
       <x:c r="S49" s="19" t="str">
         <x:v>No unsafe repeated device operation was reproduced. This is an implementation gap, not a confirmed execution defect. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
@@ -3133,10 +3135,11 @@
         <x:v>Verified (scoped)</x:v>
       </x:c>
       <x:c r="R50" s="17" t="str">
-        <x:v>Current lost-response/reload and explicit owner-safe receipt recovery pass in WSL Chrome. Native Windows packaged restart remains unverified. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+        <x:v>Current lost-response/reload and explicit owner-safe receipt recovery pass in WSL Chrome. Native Windows packaged restart remains unverified. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Mounted reload checks cover two settled, two missing and mixed receipts with independent reconciliation and unchanged unrelated pending journals. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
       </x:c>
       <x:c r="S50" s="17" t="str">
-        <x:v>This was an isolated browser/journal simulation, not a process crash of the packaged app. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+        <x:v>This was an isolated browser/journal simulation, not a process crash of the packaged app. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone. Browser admission writes require Web Locks; Windows remains unverified.</x:v>
       </x:c>
       <x:c r="T50" s="1"/>
     </x:row>
@@ -5113,7 +5116,8 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="R83" s="19" t="str">
-        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.
+Review correction: Original message ID and annotation payload remain attached to the exact retained raw evidence through same-request retry. Annotation feature verdict remains scoped/partial. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
       </x:c>
       <x:c r="S83" s="19" t="str">
         <x:v>A successful annotation is saved, but stale-result rejection, discard and save-failure paths are not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
@@ -6613,7 +6617,8 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="R108" s="17" t="str">
-        <x:v>Current local storage, response-loss, cancellation and persistence-failure fixtures preserve draft/evidence and explicit review. Provider-specific errors remain mocked; no live reachability proof. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+        <x:v>Current local storage, response-loss, cancellation and persistence-failure fixtures preserve draft/evidence and explicit review. Provider-specific errors remain mocked; no live reachability proof. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Stale snapshot is rejected without overwriting the newer draft. Explicit multi-chat recovery no longer locks out both conversations. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
       </x:c>
       <x:c r="S108" s="17" t="str">
         <x:v>Only the creation transaction/reload/retry path was fixed and tested in this batch. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
@@ -7513,10 +7518,11 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="R123" s="15" t="str">
-        <x:v>Active API enforces serial capacity; current browser waiting/draft fixture and queue checks supplement prior evidence. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+        <x:v>Active API enforces serial capacity; current browser waiting/draft fixture and queue checks supplement prior evidence. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: A genuinely live other-tab writer retains its Web Lock and completes successfully; foreign review is read-only until it finishes. Global backend serial admission remains. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
       </x:c>
       <x:c r="S123" s="15" t="str">
-        <x:v>Full serial multi-conversation queue UI was not exercised in this bounded run. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+        <x:v>Full serial multi-conversation queue UI was not exercised in this bounded run. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone. Browser admission writes require Web Locks; Windows remains unverified.</x:v>
       </x:c>
       <x:c r="T123" s="1"/>
     </x:row>
@@ -7633,7 +7639,8 @@
         <x:v>Verified (scoped)</x:v>
       </x:c>
       <x:c r="R125" s="15" t="str">
-        <x:v>Current scoped receipt and raw-run readback preserve original run/request/chat provenance and exact output. Evidence and admission settlement are distinct. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+        <x:v>Current scoped receipt and raw-run readback preserve original run/request/chat provenance and exact output. Evidence and admission settlement are distinct. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Captured event/evidence payloads survive reconciliation; repeated identical capture entries are deduplicated. Evidence-versus-receipt ambiguity remains a nonblocking limitation. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
       </x:c>
       <x:c r="S125" s="15" t="str">
         <x:v>Existing local records only; no new provider/device run, service restart or cross-device durability test. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
@@ -8471,7 +8478,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R3b91acc2d02d4683"/>
+    <x:tablePart ns1:id="R3b91acc2d02d4683"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add bounded clarification waiting and same-run continuation
</commit_message>
<xml_diff>
--- a/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
+++ b/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
@@ -2711,13 +2711,13 @@
         <x:v>A0; server/runtime source review; polished.js:193-255,380-422; intentgraph/server.cjs:206-285</x:v>
       </x:c>
       <x:c r="Q43" s="19" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="R43" s="19" t="str">
-        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+        <x:v>2026-09-19 clarification: One structured question, one bounded answer and one same-run read-only continuation implemented. Scoped API, state and mounted tests cover double-click, stale/cross-tab/cross-run answers, reload, cancellation, response loss and storage failure. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
       </x:c>
       <x:c r="S43" s="19" t="str">
-        <x:v>No external approval or device action was invoked. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+        <x:v>General approval is absent. Independent review and owner UI approval remain pending; Windows and live provider/device behavior are unverified. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
       </x:c>
       <x:c r="T43" s="1"/>
     </x:row>
@@ -2774,10 +2774,10 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="R44" s="17" t="str">
-        <x:v>Existing Plan/Inspect and allowlist tests pass; browser Plan fixture uses the same saved mode on retries. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+        <x:v>2026-09-19 clarification: Injected-model Plan clarification and hostile continuation execute with zero tools; malicious tool-bearing output fails closed. Same-run mode/provider tests and existing Inspect allowlist regressions pass. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
       </x:c>
       <x:c r="S44" s="17" t="str">
-        <x:v>The current fixture did not prove backend no-tools enforcement for every plan request. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+        <x:v>No state-changing permission is added. Live provider/device and native Windows validation remain outside; this is not full-product acceptance. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
       </x:c>
       <x:c r="T44" s="1"/>
     </x:row>
@@ -2954,10 +2954,10 @@
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="R47" s="19" t="str">
-        <x:v>Global serial admission retained. Parallel execution remains Missing. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+        <x:v>2026-09-19 clarification: Waiting explicitly retains the global serial slot; another conversation keeps its draft and links to the waiting conversation. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
       </x:c>
       <x:c r="S47" s="19" t="str">
-        <x:v>No concurrent provider/device calls were made. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+        <x:v>Parallel execution remains excluded and unimplemented. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
       </x:c>
       <x:c r="T47" s="1"/>
     </x:row>

</xml_diff>

<commit_message>
Preserve clarification runtime limits, drafts and refresh focus
</commit_message>
<xml_diff>
--- a/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
+++ b/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
@@ -2714,10 +2714,10 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="R43" s="19" t="str">
-        <x:v>2026-09-19 clarification: One structured question, one bounded answer and one same-run read-only continuation implemented. Scoped API, state and mounted tests cover double-click, stale/cross-tab/cross-run answers, reload, cancellation, response loss and storage failure. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
+        <x:v>2026-09-19 review corrections: F1–F3 corrections retain bounded live model/tool context, six-call budget and diagnostic attempts; persist drafts on edits before Continue and after rejection; restore Refresh focus and announce status. Actual LangChain/runtime and mounted reload/focus regressions pass. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
       </x:c>
       <x:c r="S43" s="19" t="str">
-        <x:v>General approval is absent. Independent review and owner UI approval remain pending; Windows and live provider/device behavior are unverified. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
+        <x:v>General approval is absent. Independent re-review of corrections and owner UI approval remain pending; Windows and live provider/device behavior are unverified. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
       </x:c>
       <x:c r="T43" s="1"/>
     </x:row>
@@ -2774,10 +2774,10 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="R44" s="17" t="str">
-        <x:v>2026-09-19 clarification: Injected-model Plan clarification and hostile continuation execute with zero tools; malicious tool-bearing output fails closed. Same-run mode/provider tests and existing Inspect allowlist regressions pass. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
+        <x:v>2026-09-19 review corrections: Both clarification segments share the original model, six-call budget and diagnostic-attempt set. An UNKNOWN diagnostic cannot be retried after clarification. Actual LangChain Plan continuation rejects hostile tool output with zero device calls. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
       </x:c>
       <x:c r="S44" s="17" t="str">
-        <x:v>No state-changing permission is added. Live provider/device and native Windows validation remain outside; this is not full-product acceptance. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
+        <x:v>No state-changing permission or restart checkpoint is added. Live provider/device and native Windows validation remain outside; this is not full-product acceptance. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
       </x:c>
       <x:c r="T44" s="1"/>
     </x:row>

</xml_diff>

<commit_message>
feat(intentgraph): add durable chat admission and bounded clarification (#1)
* Persist serial chat admission and fence duplicate dispatch

* Keep browser submission identity through interruption and recovery

* Record admission evidence and preserve scoped feature verdicts

* Propose clarification flow and explicit approval decisions

* Reconcile pending chats independently and retain retry result identity

* Add bounded clarification waiting and same-run continuation

* Preserve clarification runtime limits, drafts and refresh focus

* no-mistakes(review): Fix pending draft persistence and guard workspace restores

* no-mistakes(test): Protect live writer completion from foreign navigation saves

* no-mistakes(test): Serialize same-tab saves to prevent false writer warnings

* no-mistakes(document): Reconcile clarification documentation and delivery status

---------

Co-authored-by: Codex <codex@localhost>
</commit_message>
<xml_diff>
--- a/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
+++ b/outputs/01a0a3bc-a376-74e1-8d48-e4029c2cb5a2/Aven-UI-UX-Feature-Register.xlsx
@@ -188,9 +188,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AvenFeatures" displayName="AvenFeatures" ref="A10:P125" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A10:P125"/>
-  <x:tableColumns count="16">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AvenFeatures" displayName="AvenFeatures" ref="A10:S125" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A10:S125"/>
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
     <x:tableColumn id="3" name="Feature"/>
@@ -207,6 +207,9 @@
     <x:tableColumn id="14" name="Delivery"/>
     <x:tableColumn id="15" name="Decision"/>
     <x:tableColumn id="16" name="Evidence"/>
+    <x:tableColumn id="17" name="Effective verdict 2026-09-19"/>
+    <x:tableColumn id="18" name="Admission evidence 2026-09-19"/>
+    <x:tableColumn id="19" name="Remaining scope / limits"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -404,7 +407,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF253448"/>
   </x:sheetPr>
@@ -426,6 +429,9 @@
     <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="46" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="29" customWidth="1"/>
+    <x:col min="18" max="18" width="72" customWidth="1"/>
+    <x:col min="19" max="19" width="65" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -651,7 +657,9 @@
       <x:c r="T8" s="1"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="1"/>
+      <x:c r="A9" s="1" t="str">
+        <x:v>19 September 2026: Q–S contain effective scoped verdicts and admission evidence. A–P and the summary above remain dated history. Counts: 37 scoped Verified, 57 Partial, 3 Unverified, 14 Missing, 4 Deferred; owner approval is separate. Independent-review recovery corrections are appended in R; verdict counts are unchanged.</x:v>
+      </x:c>
       <x:c r="B9" s="1"/>
       <x:c r="C9" s="1"/>
       <x:c r="D9" s="1"/>
@@ -721,9 +729,15 @@
       <x:c r="P10" s="8" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="Q10" s="1"/>
-      <x:c r="R10" s="1"/>
-      <x:c r="S10" s="1"/>
+      <x:c r="Q10" s="8" t="str">
+        <x:v>Effective verdict 2026-09-19</x:v>
+      </x:c>
+      <x:c r="R10" s="8" t="str">
+        <x:v>Admission evidence 2026-09-19</x:v>
+      </x:c>
+      <x:c r="S10" s="8" t="str">
+        <x:v>Remaining scope / limits</x:v>
+      </x:c>
       <x:c r="T10" s="1"/>
     </x:row>
     <x:row r="11" ht="117" customHeight="1">
@@ -775,9 +789,15 @@
       <x:c r="P11" s="15" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q11" s="1"/>
-      <x:c r="R11" s="1"/>
-      <x:c r="S11" s="1"/>
+      <x:c r="Q11" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R11" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S11" s="15" t="str">
+        <x:v>No substantive gap in the original browser interaction slice; assistive-technology and owner visual certification remain outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T11" s="1"/>
     </x:row>
     <x:row r="12" ht="117" customHeight="1">
@@ -829,9 +849,15 @@
       <x:c r="P12" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q12" s="1"/>
-      <x:c r="R12" s="1"/>
-      <x:c r="S12" s="1"/>
+      <x:c r="Q12" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R12" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S12" s="17" t="str">
+        <x:v>Agreed desktop-width matrix beyond 390px is untested, so full overflow coverage is incomplete. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T12" s="1"/>
     </x:row>
     <x:row r="13" ht="102" customHeight="1">
@@ -883,9 +909,15 @@
       <x:c r="P13" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/root-identity-review.json; review-ux-pipeline.cjs --identity-only; exit 0. Isolated Chromium, owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q13" s="1"/>
-      <x:c r="R13" s="1"/>
-      <x:c r="S13" s="1"/>
+      <x:c r="Q13" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R13" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S13" s="19" t="str">
+        <x:v>No substantive gap in the original browser interaction slice; assistive-technology certification remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T13" s="1"/>
     </x:row>
     <x:row r="14" ht="87" customHeight="1">
@@ -937,9 +969,15 @@
       <x:c r="P14" s="17" t="str">
         <x:v>2026-09-15: root-identity-review.json and root-profile-desktop.png under .intentgraph/evidence/ux-fixes-2026-09-15/; browser test exit 0. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q14" s="1"/>
-      <x:c r="R14" s="1"/>
-      <x:c r="S14" s="1"/>
+      <x:c r="Q14" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R14" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S14" s="17" t="str">
+        <x:v>The evidence does not open and edit every selected profile document after rename, so document accessibility is incomplete. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T14" s="1"/>
     </x:row>
     <x:row r="15" ht="117" customHeight="1">
@@ -991,9 +1029,15 @@
       <x:c r="P15" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q15" s="1"/>
-      <x:c r="R15" s="1"/>
-      <x:c r="S15" s="1"/>
+      <x:c r="Q15" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R15" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S15" s="19" t="str">
+        <x:v>Pointer/keyboard operation and bounds pass, but row structure has no current/reference visual or structural comparison. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T15" s="1"/>
     </x:row>
     <x:row r="16" ht="117" customHeight="1">
@@ -1045,9 +1089,15 @@
       <x:c r="P16" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q16" s="1"/>
-      <x:c r="R16" s="1"/>
-      <x:c r="S16" s="1"/>
+      <x:c r="Q16" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R16" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S16" s="17" t="str">
+        <x:v>No substantive gap in the original local interaction slice; concurrent-device synchronization remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T16" s="1"/>
     </x:row>
     <x:row r="17" ht="117" customHeight="1">
@@ -1099,9 +1149,15 @@
       <x:c r="P17" s="15" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q17" s="1"/>
-      <x:c r="R17" s="1"/>
-      <x:c r="S17" s="1"/>
+      <x:c r="Q17" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R17" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S17" s="15" t="str">
+        <x:v>The seeded test proves direct/grouped history, queue and avatar reachability, but does not exercise a new-user named-conversation start path. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T17" s="1"/>
     </x:row>
     <x:row r="18" ht="117" customHeight="1">
@@ -1153,9 +1209,15 @@
       <x:c r="P18" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-fixes-2026-09-15/history-regression.json (stable coworker title after hi); .intentgraph/runtime/verify-direct-teams.cjs:8,12 Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q18" s="1"/>
-      <x:c r="R18" s="1"/>
-      <x:c r="S18" s="1"/>
+      <x:c r="Q18" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R18" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S18" s="17" t="str">
+        <x:v>No substantive gap in the original UI identity slice; the provider stream is intentionally mocked/blocked. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T18" s="1"/>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
@@ -1207,9 +1269,15 @@
       <x:c r="P19" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/local-commands.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q19" s="1"/>
-      <x:c r="R19" s="1"/>
-      <x:c r="S19" s="1"/>
+      <x:c r="Q19" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R19" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S19" s="19" t="str">
+        <x:v>No substantive gap in the tested acceptance slice; only the seeded narrow width and title matrix were exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T19" s="1"/>
     </x:row>
     <x:row r="20" ht="72" customHeight="1">
@@ -1261,9 +1329,15 @@
       <x:c r="P20" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/project-navigation.json (pin/reload/order) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q20" s="1"/>
-      <x:c r="R20" s="1"/>
-      <x:c r="S20" s="1"/>
+      <x:c r="Q20" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R20" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S20" s="17" t="str">
+        <x:v>No substantive gap in the original local persistence slice; cross-device ordering remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T20" s="1"/>
     </x:row>
     <x:row r="21" ht="102" customHeight="1">
@@ -1315,9 +1389,15 @@
       <x:c r="P21" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (chatTitle changed; coworkerName unchanged) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q21" s="1"/>
-      <x:c r="R21" s="1"/>
-      <x:c r="S21" s="1"/>
+      <x:c r="Q21" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R21" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S21" s="19" t="str">
+        <x:v>No substantive gap in the original direct-conversation slice; broader multi-user synchronization remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T21" s="1"/>
     </x:row>
     <x:row r="22" ht="102" customHeight="1">
@@ -1369,9 +1449,15 @@
       <x:c r="P22" s="17" t="str">
         <x:v>2026-09-16: navigation.json; isolated browser test exit 0. Section boundaries, reload, failed-save atomicity and focus verified. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q22" s="1"/>
-      <x:c r="R22" s="1"/>
-      <x:c r="S22" s="1"/>
+      <x:c r="Q22" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R22" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S22" s="17" t="str">
+        <x:v>DOM separation and old-row reachability pass, but the evidence does not assert labels/affordances cannot imply coordinated execution. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T22" s="1"/>
     </x:row>
     <x:row r="23" ht="132" customHeight="1">
@@ -1423,9 +1509,15 @@
       <x:c r="P23" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/accessibility-results.json (UX096 PASS at 320/390/760/1440; page/body bounds); .intentgraph/evidence/project-navigation.json (persistent collapse) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q23" s="1"/>
-      <x:c r="R23" s="1"/>
-      <x:c r="S23" s="1"/>
+      <x:c r="Q23" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R23" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S23" s="19" t="str">
+        <x:v>No substantive gap in the original browser slice; assistive-technology certification remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T23" s="1"/>
     </x:row>
     <x:row r="24" ht="102" customHeight="1">
@@ -1477,9 +1569,15 @@
       <x:c r="P24" s="17" t="str">
         <x:v>2026-09-16: navigation.json; isolated browser test exit 0. Draft/scroll, reload, forward history, invalid storage, unsaved guards and 320-1440px bounds verified. No provider calls. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q24" s="1"/>
-      <x:c r="R24" s="1"/>
-      <x:c r="S24" s="1"/>
+      <x:c r="Q24" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R24" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S24" s="17" t="str">
+        <x:v>No substantive gap in the tested local session-history slice; cross-session/device history is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T24" s="1"/>
     </x:row>
     <x:row r="25" ht="117" customHeight="1">
@@ -1531,9 +1629,15 @@
       <x:c r="P25" s="15" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json (saved phrase, coworker/conversation filters, exact result navigation) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q25" s="1"/>
-      <x:c r="R25" s="1"/>
-      <x:c r="S25" s="1"/>
+      <x:c r="Q25" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R25" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S25" s="15" t="str">
+        <x:v>No substantive gap for the seeded known phrase; search-index breadth beyond local fixture data is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T25" s="1"/>
     </x:row>
     <x:row r="26" ht="87" customHeight="1">
@@ -1585,9 +1689,15 @@
       <x:c r="P26" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json; verify-history-navigation.cjs exit 0. Isolated mocked chat; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q26" s="1"/>
-      <x:c r="R26" s="1"/>
-      <x:c r="S26" s="1"/>
+      <x:c r="Q26" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R26" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S26" s="17" t="str">
+        <x:v>No substantive gap for the seeded duplicate-term filter result; broader external-index behavior is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T26" s="1"/>
     </x:row>
     <x:row r="27" ht="87" customHeight="1">
@@ -1639,9 +1749,15 @@
       <x:c r="P27" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/chat-interactions.json; verify-chat-interactions.cjs exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q27" s="1"/>
-      <x:c r="R27" s="1"/>
-      <x:c r="S27" s="1"/>
+      <x:c r="Q27" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R27" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S27" s="19" t="str">
+        <x:v>No substantive gap for the seeded repeated-term cycle; cross-conversation find scope is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T27" s="1"/>
     </x:row>
     <x:row r="28" ht="72" customHeight="1">
@@ -1693,9 +1809,15 @@
       <x:c r="P28" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/local-commands.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q28" s="1"/>
-      <x:c r="R28" s="1"/>
-      <x:c r="S28" s="1"/>
+      <x:c r="Q28" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R28" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S28" s="17" t="str">
+        <x:v>No substantive gap in the tested current-chat palette flow; OS-level shortcut conflicts remain outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T28" s="1"/>
     </x:row>
     <x:row r="29" ht="102" customHeight="1">
@@ -1747,9 +1869,15 @@
       <x:c r="P29" s="15" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (emptyDisabled=true, multilineHeld=true, imeHeld=true, calls=0) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q29" s="1"/>
-      <x:c r="R29" s="1"/>
-      <x:c r="S29" s="1"/>
+      <x:c r="Q29" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R29" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S29" s="15" t="str">
+        <x:v>IME composition was not simulated. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T29" s="1"/>
     </x:row>
     <x:row r="30" ht="102" customHeight="1">
@@ -1801,9 +1929,15 @@
       <x:c r="P30" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-pipeline-2026-09-16/navigation.json (back/forward preserves two drafts and reload) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q30" s="1"/>
-      <x:c r="R30" s="1"/>
-      <x:c r="S30" s="1"/>
+      <x:c r="Q30" s="17" t="str">
+        <x:v>Unverified</x:v>
+      </x:c>
+      <x:c r="R30" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S30" s="17" t="str">
+        <x:v>No fresh end-to-end evidence for independent drafts. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T30" s="1"/>
     </x:row>
     <x:row r="31" ht="102" customHeight="1">
@@ -1855,9 +1989,15 @@
       <x:c r="P31" s="19" t="str">
         <x:v>2026-09-16: attachments.json; verify-attachments-unit.cjs. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q31" s="1"/>
-      <x:c r="R31" s="1"/>
-      <x:c r="S31" s="1"/>
+      <x:c r="Q31" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R31" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S31" s="19" t="str">
+        <x:v>Fresh check did not inspect request context or unsupported-file pre-send behavior. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T31" s="1"/>
     </x:row>
     <x:row r="32" ht="72" customHeight="1">
@@ -1909,9 +2049,15 @@
       <x:c r="P32" s="17" t="str">
         <x:v>2026-09-16: attachments.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q32" s="1"/>
-      <x:c r="R32" s="1"/>
-      <x:c r="S32" s="1"/>
+      <x:c r="Q32" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R32" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S32" s="17" t="str">
+        <x:v>Drag/drop and clipboard paths were not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T32" s="1"/>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
@@ -1963,9 +2109,15 @@
       <x:c r="P33" s="19" t="str">
         <x:v>polished.html; polished.js; polished.js:213-265,408-437</x:v>
       </x:c>
-      <x:c r="Q33" s="1"/>
-      <x:c r="R33" s="1"/>
-      <x:c r="S33" s="1"/>
+      <x:c r="Q33" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R33" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S33" s="19" t="str">
+        <x:v>No provider, device, or credential calls were made by this audit. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T33" s="1"/>
     </x:row>
     <x:row r="34" ht="87" customHeight="1">
@@ -2017,9 +2169,15 @@
       <x:c r="P34" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/chat-interactions.json; verify-chat-interactions.cjs exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q34" s="1"/>
-      <x:c r="R34" s="1"/>
-      <x:c r="S34" s="1"/>
+      <x:c r="Q34" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R34" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S34" s="17" t="str">
+        <x:v>No substantive gap in the tested reply/cancel flow; the fixture used a mouse path only. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T34" s="1"/>
     </x:row>
     <x:row r="35" ht="72" customHeight="1">
@@ -2071,9 +2229,15 @@
       <x:c r="P35" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/edit-rendering.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q35" s="1"/>
-      <x:c r="R35" s="1"/>
-      <x:c r="S35" s="1"/>
+      <x:c r="Q35" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R35" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S35" s="19" t="str">
+        <x:v>No device command execution was permitted or tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T35" s="1"/>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
@@ -2125,9 +2289,15 @@
       <x:c r="P36" s="17" t="str">
         <x:v>polished.html composer; polished.js:213-265,408-437</x:v>
       </x:c>
-      <x:c r="Q36" s="1"/>
-      <x:c r="R36" s="1"/>
-      <x:c r="S36" s="1"/>
+      <x:c r="Q36" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R36" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S36" s="17" t="str">
+        <x:v>Microphone/device APIs were intentionally not called. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T36" s="1"/>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
@@ -2179,9 +2349,15 @@
       <x:c r="P37" s="19" t="str">
         <x:v>A0 Settings Models; agent-runtime.cjs; polished.js:213-265,408-437</x:v>
       </x:c>
-      <x:c r="Q37" s="1"/>
-      <x:c r="R37" s="1"/>
-      <x:c r="S37" s="1"/>
+      <x:c r="Q37" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R37" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S37" s="19" t="str">
+        <x:v>No real provider call was attempted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T37" s="1"/>
     </x:row>
     <x:row r="38" ht="117" customHeight="1">
@@ -2233,9 +2409,15 @@
       <x:c r="P38" s="21" t="str">
         <x:v>2026-09-16: preservation audit PASS. isolated run `node .intentgraph/runtime/verify-agent-stream-ui.cjs`; .intentgraph/evidence/chat-polish.json (one terminal despite duplicate event/final) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q38" s="1"/>
-      <x:c r="R38" s="1"/>
-      <x:c r="S38" s="1"/>
+      <x:c r="Q38" s="21" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R38" s="21" t="str">
+        <x:v>Current API and browser reconcile one final result after lost response/reload; exact 15-line code remains collapsed and intact. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S38" s="21" t="str">
+        <x:v>The stream was locally fulfilled; provider behavior and reconnects were not tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T38" s="1"/>
     </x:row>
     <x:row r="39" ht="87" customHeight="1">
@@ -2287,9 +2469,15 @@
       <x:c r="P39" s="19" t="str">
         <x:v>2026-09-16: verify-queue-terminal.cjs 4/4; run-durability.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q39" s="1"/>
-      <x:c r="R39" s="1"/>
-      <x:c r="S39" s="1"/>
+      <x:c r="Q39" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R39" s="19" t="str">
+        <x:v>Current Stop fixture preserves UNKNOWN and pauses queued work. Remote cancellation is not asserted. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S39" s="19" t="str">
+        <x:v>No real remote request or device command was stopped. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T39" s="1"/>
     </x:row>
     <x:row r="40" ht="132" customHeight="1">
@@ -2341,9 +2529,16 @@
       <x:c r="P40" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (storage failure: 0 calls, queue retained; recovery: 1 call); .intentgraph/runtime/verify-queue-terminal.cjs:49-75 Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q40" s="1"/>
-      <x:c r="R40" s="1"/>
-      <x:c r="S40" s="1"/>
+      <x:c r="Q40" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R40" s="17" t="str">
+        <x:v>Stable saved identities and backend duplicate suppression; current browser FIFO and explicit paused-queue checks. Broader crash-at-every-queue-boundary coverage remains partial. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Mounted three-turn FIFO dispatches once per identity after writer-lock release; paused queues survive independent pending-chat recovery. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
+      </x:c>
+      <x:c r="S40" s="17" t="str">
+        <x:v>Order and duplicate-submission behavior were not freshly exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T40" s="1"/>
     </x:row>
     <x:row r="41" ht="87" customHeight="1">
@@ -2395,9 +2590,15 @@
       <x:c r="P41" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/runtime/verify-queue-terminal.cjs:49-75,120-128 (FIFO/edit/remove/resume/reload pause) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q41" s="1"/>
-      <x:c r="R41" s="1"/>
-      <x:c r="S41" s="1"/>
+      <x:c r="Q41" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R41" s="19" t="str">
+        <x:v>Current queue survives Stop/review and resumes explicitly; this milestone does not freshly exercise every edit/remove/reorder variant. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S41" s="19" t="str">
+        <x:v>Resume and exactly-once dispatch were not tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T41" s="1"/>
     </x:row>
     <x:row r="42" ht="132" customHeight="1">
@@ -2449,9 +2650,15 @@
       <x:c r="P42" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. 25/25 local fixture tests passed, including `intentgraph/steering.test.cjs:166-191` (next model boundary, applied once); .intentgraph/runtime/verify-queue-terminal.cjs:77-118 Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q42" s="1"/>
-      <x:c r="R42" s="1"/>
-      <x:c r="S42" s="1"/>
+      <x:c r="Q42" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R42" s="17" t="str">
+        <x:v>Existing active steering tests pass unchanged; receipt identity does not replace steering tokens or authorize new work. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S42" s="17" t="str">
+        <x:v>Unit coverage does not prove the browser UI flow. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T42" s="1"/>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
@@ -2503,9 +2710,15 @@
       <x:c r="P43" s="19" t="str">
         <x:v>A0; server/runtime source review; polished.js:193-255,380-422; intentgraph/server.cjs:206-285</x:v>
       </x:c>
-      <x:c r="Q43" s="1"/>
-      <x:c r="R43" s="1"/>
-      <x:c r="S43" s="1"/>
+      <x:c r="Q43" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R43" s="19" t="str">
+        <x:v>2026-09-19 review corrections: F1–F3 corrections retain bounded live model/tool context, six-call budget and diagnostic attempts; persist drafts on edits before Continue and after rejection; restore Refresh focus and announce status. Actual LangChain/runtime and mounted reload/focus regressions pass. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
+      </x:c>
+      <x:c r="S43" s="19" t="str">
+        <x:v>General approval is absent. Independent re-review of corrections and owner UI approval remain pending; Windows and live provider/device behavior are unverified. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
+      </x:c>
       <x:c r="T43" s="1"/>
     </x:row>
     <x:row r="44" ht="87" customHeight="1">
@@ -2557,9 +2770,15 @@
       <x:c r="P44" s="17" t="str">
         <x:v>2026-09-16: verify-chat-modes.cjs and modes-ui.json passed; malicious tool-call fixture invokes no sandbox. No live provider call.</x:v>
       </x:c>
-      <x:c r="Q44" s="1"/>
-      <x:c r="R44" s="1"/>
-      <x:c r="S44" s="1"/>
+      <x:c r="Q44" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R44" s="17" t="str">
+        <x:v>2026-09-19 review corrections: Both clarification segments share the original model, six-call budget and diagnostic-attempt set. An UNKNOWN diagnostic cannot be retried after clarification. Actual LangChain Plan continuation rejects hostile tool output with zero device calls. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
+      </x:c>
+      <x:c r="S44" s="17" t="str">
+        <x:v>No state-changing permission or restart checkpoint is added. Live provider/device and native Windows validation remain outside; this is not full-product acceptance. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
+      </x:c>
       <x:c r="T44" s="1"/>
     </x:row>
     <x:row r="45" ht="102" customHeight="1">
@@ -2611,9 +2830,15 @@
       <x:c r="P45" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/runtime/verify-queue-terminal.cjs:77-118 (tool input/result/status/raw output distinct); isolated stream UI passed Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q45" s="1"/>
-      <x:c r="R45" s="1"/>
-      <x:c r="S45" s="1"/>
+      <x:c r="Q45" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R45" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S45" s="19" t="str">
+        <x:v>No substantive gap in the saved transcript representation; provider-stream coverage remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T45" s="1"/>
     </x:row>
     <x:row r="46" ht="87" customHeight="1">
@@ -2665,9 +2890,15 @@
       <x:c r="P46" s="17" t="str">
         <x:v>2026-09-16: run-recovery.json; run-durability.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q46" s="1"/>
-      <x:c r="R46" s="1"/>
-      <x:c r="S46" s="1"/>
+      <x:c r="Q46" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R46" s="17" t="str">
+        <x:v>Unknown/cancellation/persistence failures cannot be promoted to success; elapsed UI behavior retains existing implementation. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S46" s="17" t="str">
+        <x:v>Elapsed timing itself was not asserted by the fresh harness. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T46" s="1"/>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
@@ -2719,9 +2950,15 @@
       <x:c r="P47" s="19" t="str">
         <x:v>server.cjs chatPending; architecture.json; polished.js:193-255,380-422; intentgraph/server.cjs:206-285</x:v>
       </x:c>
-      <x:c r="Q47" s="1"/>
-      <x:c r="R47" s="1"/>
-      <x:c r="S47" s="1"/>
+      <x:c r="Q47" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R47" s="19" t="str">
+        <x:v>2026-09-19 clarification: Waiting explicitly retains the global serial slot; another conversation keeps its draft and links to the waiting conversation. Evidence: docs/evidence/clarification-2026-09-19/verification.json</x:v>
+      </x:c>
+      <x:c r="S47" s="19" t="str">
+        <x:v>Parallel execution remains excluded and unimplemented. Existing evidence-versus-receipt ambiguity and Windows uncertainty remain documented.</x:v>
+      </x:c>
       <x:c r="T47" s="1"/>
     </x:row>
     <x:row r="48" ht="87" customHeight="1">
@@ -2773,9 +3010,15 @@
       <x:c r="P48" s="17" t="str">
         <x:v>2026-09-16: run-recovery.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q48" s="1"/>
-      <x:c r="R48" s="1"/>
-      <x:c r="S48" s="1"/>
+      <x:c r="Q48" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R48" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S48" s="17" t="str">
+        <x:v>Unknown-usage branch and model-mismatch case were not tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T48" s="1"/>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
@@ -2827,9 +3070,16 @@
       <x:c r="P49" s="19" t="str">
         <x:v>polished.js request errors; server.cjs; polished.js:193-255,380-422; intentgraph/server.cjs:206-285</x:v>
       </x:c>
-      <x:c r="Q49" s="1"/>
-      <x:c r="R49" s="1"/>
-      <x:c r="S49" s="1"/>
+      <x:c r="Q49" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R49" s="19" t="str">
+        <x:v>Current storage/API/browser replay uses the same receipt and never dispatches automatically. Partial: no live device or checkpoint resumption validation. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Outage -&gt; missing receipt -&gt; successful Retry saved request updates one original message and retains timestamp, annotations and raw capture; no contradictory UNKNOWN/SUCCESS pair. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
+      </x:c>
+      <x:c r="S49" s="19" t="str">
+        <x:v>No unsafe repeated device operation was reproduced. This is an implementation gap, not a confirmed execution defect. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T49" s="1"/>
     </x:row>
     <x:row r="50" ht="87" customHeight="1">
@@ -2881,9 +3131,16 @@
       <x:c r="P50" s="17" t="str">
         <x:v>2026-09-16: run-recovery.json; run-durability.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q50" s="1"/>
-      <x:c r="R50" s="1"/>
-      <x:c r="S50" s="1"/>
+      <x:c r="Q50" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R50" s="17" t="str">
+        <x:v>Current lost-response/reload and explicit owner-safe receipt recovery pass in WSL Chrome. Native Windows packaged restart remains unverified. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Mounted reload checks cover two settled, two missing and mixed receipts with independent reconciliation and unchanged unrelated pending journals. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
+      </x:c>
+      <x:c r="S50" s="17" t="str">
+        <x:v>This was an isolated browser/journal simulation, not a process crash of the packaged app. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone. Browser admission writes require Web Locks; Windows remains unverified.</x:v>
+      </x:c>
       <x:c r="T50" s="1"/>
     </x:row>
     <x:row r="51" ht="72" customHeight="1">
@@ -2935,9 +3192,15 @@
       <x:c r="P51" s="15" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/edit-rendering.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q51" s="1"/>
-      <x:c r="R51" s="1"/>
-      <x:c r="S51" s="1"/>
+      <x:c r="Q51" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R51" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S51" s="15" t="str">
+        <x:v>No substantive gap in the representative readability and inert-HTML slice; broader sanitizer fuzzing remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T51" s="1"/>
     </x:row>
     <x:row r="52" ht="117" customHeight="1">
@@ -2989,9 +3252,15 @@
       <x:c r="P52" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/runtime/verify-queue-terminal.cjs:77-118 (exact raw whitespace/copy); .intentgraph/evidence/ux-fixes-2026-09-15/root-review.json Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q52" s="1"/>
-      <x:c r="R52" s="1"/>
-      <x:c r="S52" s="1"/>
+      <x:c r="Q52" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R52" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S52" s="17" t="str">
+        <x:v>No substantive gap in the tested exact-copy and single-render slice; OS clipboard integration remains isolated. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T52" s="1"/>
     </x:row>
     <x:row r="53" ht="117" customHeight="1">
@@ -3043,9 +3312,15 @@
       <x:c r="P53" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (clipboard denial reports failure); .intentgraph/evidence/message-tools.json (answer/question copy) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q53" s="1"/>
-      <x:c r="R53" s="1"/>
-      <x:c r="S53" s="1"/>
+      <x:c r="Q53" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R53" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S53" s="19" t="str">
+        <x:v>No substantive gap in correct-copy and denied-clipboard feedback; OS clipboard integration remains isolated. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T53" s="1"/>
     </x:row>
     <x:row r="54" ht="87" customHeight="1">
@@ -3097,9 +3372,15 @@
       <x:c r="P54" s="17" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json; verify-history-navigation.cjs exit 0. Isolated mocked chat; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q54" s="1"/>
-      <x:c r="R54" s="1"/>
-      <x:c r="S54" s="1"/>
+      <x:c r="Q54" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R54" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S54" s="17" t="str">
+        <x:v>No substantive gap in old/new grouping and focused labels; timezone presentation matrix remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T54" s="1"/>
     </x:row>
     <x:row r="55" ht="87" customHeight="1">
@@ -3151,9 +3432,15 @@
       <x:c r="P55" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json; verify-history-navigation.cjs exit 0. Isolated mocked chat; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q55" s="1"/>
-      <x:c r="R55" s="1"/>
-      <x:c r="S55" s="1"/>
+      <x:c r="Q55" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R55" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S55" s="19" t="str">
+        <x:v>No substantive gap in the injected new-output/reading-position slice; live provider streaming is outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T55" s="1"/>
     </x:row>
     <x:row r="56" ht="132" customHeight="1">
@@ -3205,9 +3492,15 @@
       <x:c r="P56" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-fixes-2026-09-15/history-regression.json (revert no execution, undo after reload); .intentgraph/runtime/verify-edit-rendering.cjs:1-16 (queued edit disabled) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q56" s="1"/>
-      <x:c r="R56" s="1"/>
-      <x:c r="S56" s="1"/>
+      <x:c r="Q56" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R56" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S56" s="17" t="str">
+        <x:v>The busy active-run protection branch is not exercised; queued-work protection alone does not close the full acceptance. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T56" s="1"/>
     </x:row>
     <x:row r="57" ht="87" customHeight="1">
@@ -3259,9 +3552,15 @@
       <x:c r="P57" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json; verify-history-navigation.cjs exit 0. Isolated mocked chat; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q57" s="1"/>
-      <x:c r="R57" s="1"/>
-      <x:c r="S57" s="1"/>
+      <x:c r="Q57" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R57" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S57" s="19" t="str">
+        <x:v>No substantive gap in fork provenance, parent immutability and reload revisit; cross-device sync remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T57" s="1"/>
     </x:row>
     <x:row r="58" ht="87" customHeight="1">
@@ -3313,9 +3612,15 @@
       <x:c r="P58" s="17" t="str">
         <x:v>2026-09-16: run-recovery.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q58" s="1"/>
-      <x:c r="R58" s="1"/>
-      <x:c r="S58" s="1"/>
+      <x:c r="Q58" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R58" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S58" s="17" t="str">
+        <x:v>No substantive gap in the v9 live existing/missing/archived local-link slice; external URL handling remains outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T58" s="1"/>
     </x:row>
     <x:row r="59" ht="117" customHeight="1">
@@ -3367,9 +3672,15 @@
       <x:c r="P59" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q59" s="1"/>
-      <x:c r="R59" s="1"/>
-      <x:c r="S59" s="1"/>
+      <x:c r="Q59" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R59" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S59" s="19" t="str">
+        <x:v>The reaction candidate covers search, contained keyboard navigation, Escape focus return and persistence, but its isolated candidate browser run is not a fresh served v9.1 run; screen-reader, visual-reference and multi-device checks remain outside. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T59" s="1"/>
     </x:row>
     <x:row r="60" ht="132" customHeight="1">
@@ -3421,9 +3732,15 @@
       <x:c r="P60" s="21" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/project-navigation.json (archive/restore/reload and busy guard); .intentgraph/evidence/ux-fixes-2026-09-15/history-navigation.json (archived read-only) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q60" s="1"/>
-      <x:c r="R60" s="1"/>
-      <x:c r="S60" s="1"/>
+      <x:c r="Q60" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R60" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S60" s="21" t="str">
+        <x:v>The archive/restore check confirms composer state and one message, but does not deep-compare the full message/evidence payload before and after restore. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T60" s="1"/>
     </x:row>
     <x:row r="61" ht="117" customHeight="1">
@@ -3475,9 +3792,15 @@
       <x:c r="P61" s="19" t="str">
         <x:v>2026-09-15: local-data-ui.json; browser test exit 0. verify-backup-schema.cjs 9/9 passed, including private-field rejection, exact evidence, UTF-8 size boundary and interrupted-import recovery. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q61" s="1"/>
-      <x:c r="R61" s="1"/>
-      <x:c r="S61" s="1"/>
+      <x:c r="Q61" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R61" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S61" s="19" t="str">
+        <x:v>Export checks format, selected chat presence, pin metadata and token exclusion, but does not assert exact selected scope, timestamps and raw evidence comprehensively. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T61" s="1"/>
     </x:row>
     <x:row r="62" ht="117" customHeight="1">
@@ -3529,9 +3852,15 @@
       <x:c r="P62" s="17" t="str">
         <x:v>2026-09-15: local-data-ui.json; browser test exit 0. verify-backup-schema.cjs 9/9 passed, including private-field rejection, exact evidence, UTF-8 size boundary and interrupted-import recovery. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q62" s="1"/>
-      <x:c r="R62" s="1"/>
-      <x:c r="S62" s="1"/>
+      <x:c r="Q62" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R62" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S62" s="17" t="str">
+        <x:v>No substantive gap in invalid-JSON safety plus valid Add-mode preservation of unrelated work, pins and queues; the check is local-browser scoped. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T62" s="1"/>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
@@ -3583,9 +3912,15 @@
       <x:c r="P63" s="19" t="str">
         <x:v>architecture.json; polished.js persistence; polished.js:19-58,158-174,460,481</x:v>
       </x:c>
-      <x:c r="Q63" s="1"/>
-      <x:c r="R63" s="1"/>
-      <x:c r="S63" s="1"/>
+      <x:c r="Q63" s="19" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="R63" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S63" s="19" t="str">
+        <x:v>No cross-device service exists in this build. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T63" s="1"/>
     </x:row>
     <x:row r="64" ht="132" customHeight="1">
@@ -3637,9 +3972,15 @@
       <x:c r="P64" s="21" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/avatar-family-app-qa-results.json (all avatar choices/custom color/photo/migration/reload; no external requests); .intentgraph/runtime/verify-backup-schema.cjs:4,15-28 Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q64" s="1"/>
-      <x:c r="R64" s="1"/>
-      <x:c r="S64" s="1"/>
+      <x:c r="Q64" s="21" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R64" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S64" s="21" t="str">
+        <x:v>No substantive gap in legacy avatar normalization, chosen avatar persistence and reload; the check uses one legacy fixture. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T64" s="1"/>
     </x:row>
     <x:row r="65" ht="132" customHeight="1">
@@ -3691,9 +4032,15 @@
       <x:c r="P65" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/ux-fixes-2026-09-15/root-identity-review.json (profile identity/rename sync); .intentgraph/avatar-family-app-qa-results.json (long-name responsive fixture) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q65" s="1"/>
-      <x:c r="R65" s="1"/>
-      <x:c r="S65" s="1"/>
+      <x:c r="Q65" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R65" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S65" s="19" t="str">
+        <x:v>The long label remains selected-only, but only one long name is exercised and persisted reload of the saved edit is not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T65" s="1"/>
     </x:row>
     <x:row r="66" ht="87" customHeight="1">
@@ -3745,9 +4092,15 @@
       <x:c r="P66" s="17" t="str">
         <x:v>2026-09-16: pane-controls.json. Remaining scope is explicit; not marked complete.</x:v>
       </x:c>
-      <x:c r="Q66" s="1"/>
-      <x:c r="R66" s="1"/>
-      <x:c r="S66" s="1"/>
+      <x:c r="Q66" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R66" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S66" s="17" t="str">
+        <x:v>Saving and consuming the same document in a real model request were not demonstrated. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T66" s="1"/>
     </x:row>
     <x:row r="67" ht="72" customHeight="1">
@@ -3799,9 +4152,15 @@
       <x:c r="P67" s="19" t="str">
         <x:v>2026-09-16: alerts.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q67" s="1"/>
-      <x:c r="R67" s="1"/>
-      <x:c r="S67" s="1"/>
+      <x:c r="Q67" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R67" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S67" s="19" t="str">
+        <x:v>Finished enabled and muted paths pass, but waiting/error alert variants remain owned by the unintegrated automation alert core. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T67" s="1"/>
     </x:row>
     <x:row r="68" ht="70" customHeight="1">
@@ -3853,9 +4212,15 @@
       <x:c r="P68" s="17" t="str">
         <x:v>2026-09-16: accessibility-results.json UX058. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q68" s="1"/>
-      <x:c r="R68" s="1"/>
-      <x:c r="S68" s="1"/>
+      <x:c r="Q68" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R68" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S68" s="17" t="str">
+        <x:v>No substantive gap in local welcome semantics and persisted first-chat behavior; no model/provider request or cross-device storage is exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T68" s="1"/>
     </x:row>
     <x:row r="69" ht="117" customHeight="1">
@@ -3907,9 +4272,15 @@
       <x:c r="P69" s="15" t="str">
         <x:v>2026-09-15: local-data-ui.json; browser test exit 0. verify-backup-schema.cjs 9/9 passed, including private-field rejection, exact evidence, UTF-8 size boundary and interrupted-import recovery. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q69" s="1"/>
-      <x:c r="R69" s="1"/>
-      <x:c r="S69" s="1"/>
+      <x:c r="Q69" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R69" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S69" s="15" t="str">
+        <x:v>Both theme colors/readability and save/cancel pass, but persistence across a reload is not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T69" s="1"/>
     </x:row>
     <x:row r="70" ht="87" customHeight="1">
@@ -3961,9 +4332,15 @@
       <x:c r="P70" s="17" t="str">
         <x:v>2026-09-16: diagnostics-ui.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q70" s="1"/>
-      <x:c r="R70" s="1"/>
-      <x:c r="S70" s="1"/>
+      <x:c r="Q70" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R70" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S70" s="17" t="str">
+        <x:v>Local configured status is not proof of provider reachability; no credentials or provider requests were used. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T70" s="1"/>
     </x:row>
     <x:row r="71" ht="72" customHeight="1">
@@ -4015,9 +4392,15 @@
       <x:c r="P71" s="19" t="str">
         <x:v>2026-09-16: diagnostics-ui.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q71" s="1"/>
-      <x:c r="R71" s="1"/>
-      <x:c r="S71" s="1"/>
+      <x:c r="Q71" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R71" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S71" s="19" t="str">
+        <x:v>No remote adapter health check or inventory load was performed. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T71" s="1"/>
     </x:row>
     <x:row r="72" ht="102" customHeight="1">
@@ -4069,9 +4452,15 @@
       <x:c r="P72" s="17" t="str">
         <x:v>2026-09-16: verify-local-data-ui.cjs; verify-backup-schema.cjs 10 tests; attachments.json. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q72" s="1"/>
-      <x:c r="R72" s="1"/>
-      <x:c r="S72" s="1"/>
+      <x:c r="Q72" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R72" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S72" s="17" t="str">
+        <x:v>The privacy wording passes, while destructive reset/recovery behavior is not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T72" s="1"/>
     </x:row>
     <x:row r="73" ht="42" customHeight="1">
@@ -4123,9 +4512,15 @@
       <x:c r="P73" s="19" t="str">
         <x:v>A0; polished.html account-menu; polished.js:480-482</x:v>
       </x:c>
-      <x:c r="Q73" s="1"/>
-      <x:c r="R73" s="1"/>
-      <x:c r="S73" s="1"/>
+      <x:c r="Q73" s="19" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="R73" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S73" s="19" t="str">
+        <x:v>No remote identity is connected. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T73" s="1"/>
     </x:row>
     <x:row r="74" ht="87" customHeight="1">
@@ -4177,9 +4572,15 @@
       <x:c r="P74" s="17" t="str">
         <x:v>2026-09-16: diagnostics-ui.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q74" s="1"/>
-      <x:c r="R74" s="1"/>
-      <x:c r="S74" s="1"/>
+      <x:c r="Q74" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R74" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S74" s="17" t="str">
+        <x:v>Only one help entry and a successful local feedback save are checked; every-help coverage and feedback storage failure are absent. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T74" s="1"/>
     </x:row>
     <x:row r="75" ht="72" customHeight="1">
@@ -4231,9 +4632,15 @@
       <x:c r="P75" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/local-commands.json; browser test exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q75" s="1"/>
-      <x:c r="R75" s="1"/>
-      <x:c r="S75" s="1"/>
+      <x:c r="Q75" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R75" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S75" s="19" t="str">
+        <x:v>Ctrl+K and displayed shortcut text pass, but Cmd/Ctrl+F behavior and unavailable-action filtering are not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T75" s="1"/>
     </x:row>
     <x:row r="76" ht="87" customHeight="1">
@@ -4285,9 +4692,15 @@
       <x:c r="P76" s="21" t="str">
         <x:v>2026-09-16: workspace-shell.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q76" s="1"/>
-      <x:c r="R76" s="1"/>
-      <x:c r="S76" s="1"/>
+      <x:c r="Q76" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R76" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S76" s="21" t="str">
+        <x:v>Deduplication fix verified for unambiguous mirrored results; broader artifact-file capability remains partial. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T76" s="1"/>
     </x:row>
     <x:row r="77" ht="72" customHeight="1">
@@ -4339,9 +4752,15 @@
       <x:c r="P77" s="19" t="str">
         <x:v>2026-09-16: pane-controls.json. Remaining scope is explicit; not marked complete.</x:v>
       </x:c>
-      <x:c r="Q77" s="1"/>
-      <x:c r="R77" s="1"/>
-      <x:c r="S77" s="1"/>
+      <x:c r="Q77" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R77" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S77" s="19" t="str">
+        <x:v>Unavailable state passed; live browsing capability remains absent. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T77" s="1"/>
     </x:row>
     <x:row r="78" ht="87" customHeight="1">
@@ -4393,9 +4812,15 @@
       <x:c r="P78" s="17" t="str">
         <x:v>2026-09-16: pane-controls.json. Remaining scope is explicit; not marked complete.</x:v>
       </x:c>
-      <x:c r="Q78" s="1"/>
-      <x:c r="R78" s="1"/>
-      <x:c r="S78" s="1"/>
+      <x:c r="Q78" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R78" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S78" s="17" t="str">
+        <x:v>Unavailable state passed; live computer control remains absent. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T78" s="1"/>
     </x:row>
     <x:row r="79" ht="87" customHeight="1">
@@ -4447,9 +4872,15 @@
       <x:c r="P79" s="19" t="str">
         <x:v>2026-09-16: pane-controls.json. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q79" s="1"/>
-      <x:c r="R79" s="1"/>
-      <x:c r="S79" s="1"/>
+      <x:c r="Q79" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R79" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S79" s="19" t="str">
+        <x:v>One keyboard resize and focus return pass, but evidence-specific read/type room and a broader resize matrix are not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T79" s="1"/>
     </x:row>
     <x:row r="80" ht="102" customHeight="1">
@@ -4501,9 +4932,15 @@
       <x:c r="P80" s="17" t="str">
         <x:v>2026-09-16: verify-local-files.cjs 34 checks; files-shell.json 26 checks with real Web Crypto and memory-only file handles. No user disk writes. Real OS picker and owner acceptance remain unverified.</x:v>
       </x:c>
-      <x:c r="Q80" s="1"/>
-      <x:c r="R80" s="1"/>
-      <x:c r="S80" s="1"/>
+      <x:c r="Q80" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R80" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S80" s="17" t="str">
+        <x:v>No user disk writes were performed. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T80" s="1"/>
     </x:row>
     <x:row r="81" ht="42" customHeight="1">
@@ -4555,9 +4992,15 @@
       <x:c r="P81" s="19" t="str">
         <x:v>architecture.json; polished.js; polished.js:319-370</x:v>
       </x:c>
-      <x:c r="Q81" s="1"/>
-      <x:c r="R81" s="1"/>
-      <x:c r="S81" s="1"/>
+      <x:c r="Q81" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R81" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S81" s="19" t="str">
+        <x:v>Intentional scope gap. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T81" s="1"/>
     </x:row>
     <x:row r="82" ht="102" customHeight="1">
@@ -4609,9 +5052,15 @@
       <x:c r="P82" s="21" t="str">
         <x:v>2026-09-16: files-shell.json passed. Verified local file slice only; network configuration review is not claimed.</x:v>
       </x:c>
-      <x:c r="Q82" s="1"/>
-      <x:c r="R82" s="1"/>
-      <x:c r="S82" s="1"/>
+      <x:c r="Q82" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R82" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S82" s="21" t="str">
+        <x:v>No network configuration calls were made. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T82" s="1"/>
     </x:row>
     <x:row r="83" ht="87" customHeight="1">
@@ -4663,9 +5112,16 @@
       <x:c r="P83" s="19" t="str">
         <x:v>2026-09-16: evidence-shell/evidence-shell-results.json 11 checks. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q83" s="1"/>
-      <x:c r="R83" s="1"/>
-      <x:c r="S83" s="1"/>
+      <x:c r="Q83" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R83" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.
+Review correction: Original message ID and annotation payload remain attached to the exact retained raw evidence through same-request retry. Annotation feature verdict remains scoped/partial. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
+      </x:c>
+      <x:c r="S83" s="19" t="str">
+        <x:v>A successful annotation is saved, but stale-result rejection, discard and save-failure paths are not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T83" s="1"/>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
@@ -4717,9 +5173,15 @@
       <x:c r="P84" s="17" t="str">
         <x:v>intentgraph/adapters/index.cjs:462-503,570-598; polished.js:359-370</x:v>
       </x:c>
-      <x:c r="Q84" s="1"/>
-      <x:c r="R84" s="1"/>
-      <x:c r="S84" s="1"/>
+      <x:c r="Q84" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R84" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S84" s="17" t="str">
+        <x:v>No execution or provider calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T84" s="1"/>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
@@ -4771,9 +5233,15 @@
       <x:c r="P85" s="19" t="str">
         <x:v>polished.html; polished.js; intentgraph/adapters/index.cjs:462-503,570-598; polished.js:359-370</x:v>
       </x:c>
-      <x:c r="Q85" s="1"/>
-      <x:c r="R85" s="1"/>
-      <x:c r="S85" s="1"/>
+      <x:c r="Q85" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R85" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S85" s="19" t="str">
+        <x:v>No Git operation was attempted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T85" s="1"/>
     </x:row>
     <x:row r="86" ht="42" customHeight="1">
@@ -4825,9 +5293,15 @@
       <x:c r="P86" s="21" t="str">
         <x:v>polished.js:332-357; intentgraph/agent-runtime.cjs:271-338</x:v>
       </x:c>
-      <x:c r="Q86" s="1"/>
-      <x:c r="R86" s="1"/>
-      <x:c r="S86" s="1"/>
+      <x:c r="Q86" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R86" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S86" s="21" t="str">
+        <x:v>Inventory route was mocked and no device call was made. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T86" s="1"/>
     </x:row>
     <x:row r="87" ht="72" customHeight="1">
@@ -4879,9 +5353,15 @@
       <x:c r="P87" s="19" t="str">
         <x:v>2026-09-16: pane-controls.json; verify-chat-modes.cjs. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q87" s="1"/>
-      <x:c r="R87" s="1"/>
-      <x:c r="S87" s="1"/>
+      <x:c r="Q87" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R87" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S87" s="19" t="str">
+        <x:v>No live device call or enforcement backend was used. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T87" s="1"/>
     </x:row>
     <x:row r="88" ht="132" customHeight="1">
@@ -4933,9 +5413,15 @@
       <x:c r="P88" s="17" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (Markdown has run-42 and command/target); .intentgraph/evidence/ux-fixes-2026-09-15/local-data-ui.json (raw export) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q88" s="1"/>
-      <x:c r="R88" s="1"/>
-      <x:c r="S88" s="1"/>
+      <x:c r="Q88" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R88" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S88" s="17" t="str">
+        <x:v>Exact copied/exported evidence provenance across all timestamps and commands was not asserted. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T88" s="1"/>
     </x:row>
     <x:row r="89" ht="102" customHeight="1">
@@ -4987,9 +5473,15 @@
       <x:c r="P89" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. preserved-audit.json: top-level SUCCESS with nested FAILURE renders FAILURE; run state outcome precedence verified Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q89" s="1"/>
-      <x:c r="R89" s="1"/>
-      <x:c r="S89" s="1"/>
+      <x:c r="Q89" s="19" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R89" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S89" s="19" t="str">
+        <x:v>The device health conclusion is fixture-driven. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T89" s="1"/>
     </x:row>
     <x:row r="90" ht="42" customHeight="1">
@@ -5041,9 +5533,15 @@
       <x:c r="P90" s="17" t="str">
         <x:v>architecture.json; intentgraph/agent-runtime.cjs:203-214,271-415</x:v>
       </x:c>
-      <x:c r="Q90" s="1"/>
-      <x:c r="R90" s="1"/>
-      <x:c r="S90" s="1"/>
+      <x:c r="Q90" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R90" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S90" s="17" t="str">
+        <x:v>No state-changing workflow is present to exercise. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T90" s="1"/>
     </x:row>
     <x:row r="91" ht="87" customHeight="1">
@@ -5095,9 +5593,15 @@
       <x:c r="P91" s="19" t="str">
         <x:v>2026-09-16: evidence-shell/evidence-shell-results.json; verify-evidence-tools.cjs. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q91" s="1"/>
-      <x:c r="R91" s="1"/>
-      <x:c r="S91" s="1"/>
+      <x:c r="Q91" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R91" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S91" s="19" t="str">
+        <x:v>The comparison UI and timestamp labeling across different runs were not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T91" s="1"/>
     </x:row>
     <x:row r="92" ht="42" customHeight="1">
@@ -5149,9 +5653,15 @@
       <x:c r="P92" s="17" t="str">
         <x:v>Runtime/output verification needed; intentgraph/agent-runtime.cjs:203-214,271-415</x:v>
       </x:c>
-      <x:c r="Q92" s="1"/>
-      <x:c r="R92" s="1"/>
-      <x:c r="S92" s="1"/>
+      <x:c r="Q92" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R92" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S92" s="17" t="str">
+        <x:v>No topology data contract or renderer in Aven shell. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T92" s="1"/>
     </x:row>
     <x:row r="93" ht="87" customHeight="1">
@@ -5203,9 +5713,15 @@
       <x:c r="P93" s="15" t="str">
         <x:v>2026-09-16: workspace-shell.json; verify-workspace-tools.cjs 30 checks. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q93" s="1"/>
-      <x:c r="R93" s="1"/>
-      <x:c r="S93" s="1"/>
+      <x:c r="Q93" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R93" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S93" s="15" t="str">
+        <x:v>Only the empty Feed explanation is exercised; populated entries opening their distinct saved runs are not. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T93" s="1"/>
     </x:row>
     <x:row r="94" ht="87" customHeight="1">
@@ -5257,9 +5773,15 @@
       <x:c r="P94" s="17" t="str">
         <x:v>2026-09-16: workspace-shell.json; verify-workspace-tools.cjs 30 checks. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q94" s="1"/>
-      <x:c r="R94" s="1"/>
-      <x:c r="S94" s="1"/>
+      <x:c r="Q94" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R94" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S94" s="17" t="str">
+        <x:v>No substantive gap in local idea add/save/reload/archive/restore behavior; no remote persistence is exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T94" s="1"/>
     </x:row>
     <x:row r="95" ht="87" customHeight="1">
@@ -5311,9 +5833,15 @@
       <x:c r="P95" s="19" t="str">
         <x:v>2026-09-16: verify-workspace-tools.cjs 30 checks; workspace-shell.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q95" s="1"/>
-      <x:c r="R95" s="1"/>
-      <x:c r="S95" s="1"/>
+      <x:c r="Q95" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R95" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S95" s="19" t="str">
+        <x:v>The child module check only inspected source text. Completion, persistence and invalid-evidence rejection were not behaviorally tested. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T95" s="1"/>
     </x:row>
     <x:row r="96" ht="42" customHeight="1">
@@ -5365,9 +5893,15 @@
       <x:c r="P96" s="17" t="str">
         <x:v>polished.html; server.cjs; polished.js:434-449; intentgraph/ui/index.html:7-8</x:v>
       </x:c>
-      <x:c r="Q96" s="1"/>
-      <x:c r="R96" s="1"/>
-      <x:c r="S96" s="1"/>
+      <x:c r="Q96" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R96" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S96" s="17" t="str">
+        <x:v>No scheduler surface exists. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T96" s="1"/>
     </x:row>
     <x:row r="97" ht="72" customHeight="1">
@@ -5419,9 +5953,15 @@
       <x:c r="P97" s="19" t="str">
         <x:v>2026-09-16: alerts.json. Implemented slice verified; full feature remains pending.</x:v>
       </x:c>
-      <x:c r="Q97" s="1"/>
-      <x:c r="R97" s="1"/>
-      <x:c r="S97" s="1"/>
+      <x:c r="Q97" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R97" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S97" s="19" t="str">
+        <x:v>The enabled preference and finished-result path are covered through UX-057, but waiting/error variants and duplicate visible-alert suppression are not. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T97" s="1"/>
     </x:row>
     <x:row r="98" ht="42" customHeight="1">
@@ -5473,9 +6013,15 @@
       <x:c r="P98" s="17" t="str">
         <x:v>polished.html plugins pane; polished.js:434-449; intentgraph/ui/index.html:7-8</x:v>
       </x:c>
-      <x:c r="Q98" s="1"/>
-      <x:c r="R98" s="1"/>
-      <x:c r="S98" s="1"/>
+      <x:c r="Q98" s="17" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R98" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S98" s="17" t="str">
+        <x:v>Local fixtures only; no provider/device calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T98" s="1"/>
     </x:row>
     <x:row r="99" ht="42" customHeight="1">
@@ -5527,9 +6073,15 @@
       <x:c r="P99" s="19" t="str">
         <x:v>polished.js documents; runtime; polished.js:434-449; intentgraph/ui/index.html:7-8</x:v>
       </x:c>
-      <x:c r="Q99" s="1"/>
-      <x:c r="R99" s="1"/>
-      <x:c r="S99" s="1"/>
+      <x:c r="Q99" s="19" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R99" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S99" s="19" t="str">
+        <x:v>Local documents exist, but the requested reusable workflow capability is absent. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T99" s="1"/>
     </x:row>
     <x:row r="100" ht="42" customHeight="1">
@@ -5581,9 +6133,15 @@
       <x:c r="P100" s="17" t="str">
         <x:v>architecture.json; polished.js:434-449; intentgraph/ui/index.html:7-8</x:v>
       </x:c>
-      <x:c r="Q100" s="1"/>
-      <x:c r="R100" s="1"/>
-      <x:c r="S100" s="1"/>
+      <x:c r="Q100" s="17" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="R100" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S100" s="17" t="str">
+        <x:v>Deferred by user decision. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T100" s="1"/>
     </x:row>
     <x:row r="101" ht="72" customHeight="1">
@@ -5635,9 +6193,15 @@
       <x:c r="P101" s="15" t="str">
         <x:v>2026-09-16: accessibility-results.json; pane-controls.json. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q101" s="1"/>
-      <x:c r="R101" s="1"/>
-      <x:c r="S101" s="1"/>
+      <x:c r="Q101" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R101" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S101" s="15" t="str">
+        <x:v>Plus/settings keyboard paths pass, but all visible controls, full logical order, trap detection and every Escape return are not covered. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T101" s="1"/>
     </x:row>
     <x:row r="102" ht="72" customHeight="1">
@@ -5689,9 +6253,15 @@
       <x:c r="P102" s="17" t="str">
         <x:v>2026-09-16: accessibility-results.json UX092; no full WCAG conformance claim. Local isolated checks passed; owner acceptance separate.</x:v>
       </x:c>
-      <x:c r="Q102" s="1"/>
-      <x:c r="R102" s="1"/>
-      <x:c r="S102" s="1"/>
+      <x:c r="Q102" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R102" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S102" s="17" t="str">
+        <x:v>Representative ARIA roles/names and selected state pass, but there is no screen-reader run covering every action, coworker and active-run state. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T102" s="1"/>
     </x:row>
     <x:row r="103" ht="87" customHeight="1">
@@ -5743,9 +6313,15 @@
       <x:c r="P103" s="19" t="str">
         <x:v>2026-09-16: accessibility-results.json; scoped checks, not a full WCAG conformance claim. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q103" s="1"/>
-      <x:c r="R103" s="1"/>
-      <x:c r="S103" s="1"/>
+      <x:c r="Q103" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R103" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S103" s="19" t="str">
+        <x:v>One answer contrast measurement and 200% narrow overflow check pass, but all controls and a broader narrow/reflow matrix are not measured. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T103" s="1"/>
     </x:row>
     <x:row r="104" ht="72" customHeight="1">
@@ -5797,9 +6373,15 @@
       <x:c r="P104" s="17" t="str">
         <x:v>2026-09-16: accessibility-results.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q104" s="1"/>
-      <x:c r="R104" s="1"/>
-      <x:c r="S104" s="1"/>
+      <x:c r="Q104" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R104" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S104" s="17" t="str">
+        <x:v>Decorative animation is disabled under reduced motion, but state-changing interactions under the preference are not exercised. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T104" s="1"/>
     </x:row>
     <x:row r="105" ht="72" customHeight="1">
@@ -5851,9 +6433,15 @@
       <x:c r="P105" s="19" t="str">
         <x:v>2026-09-16: accessibility-results.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q105" s="1"/>
-      <x:c r="R105" s="1"/>
-      <x:c r="S105" s="1"/>
+      <x:c r="Q105" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R105" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S105" s="19" t="str">
+        <x:v>Touch target sizes pass, but hover menu bounds, close behavior and focus restoration are not covered by this quality check. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T105" s="1"/>
     </x:row>
     <x:row r="106" ht="72" customHeight="1">
@@ -5905,9 +6493,15 @@
       <x:c r="P106" s="17" t="str">
         <x:v>2026-09-16: accessibility-results.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q106" s="1"/>
-      <x:c r="R106" s="1"/>
-      <x:c r="S106" s="1"/>
+      <x:c r="Q106" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R106" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S106" s="17" t="str">
+        <x:v>A 320px pane open/close and containment check passes, but desktop/zoomed controls and deliberate table scrolling are not covered. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T106" s="1"/>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
@@ -5959,9 +6553,15 @@
       <x:c r="P107" s="19" t="str">
         <x:v>A0 Feed, Artifacts, Settings; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q107" s="1"/>
-      <x:c r="R107" s="1"/>
-      <x:c r="S107" s="1"/>
+      <x:c r="Q107" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R107" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S107" s="19" t="str">
+        <x:v>Unavailable context is truthful, but the evidence does not enumerate every visible action and its real result/unavailable explanation. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T107" s="1"/>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
@@ -6013,9 +6613,16 @@
       <x:c r="P108" s="17" t="str">
         <x:v>polished.js request handlers; server.cjs; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q108" s="1"/>
-      <x:c r="R108" s="1"/>
-      <x:c r="S108" s="1"/>
+      <x:c r="Q108" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R108" s="17" t="str">
+        <x:v>Current local storage, response-loss, cancellation and persistence-failure fixtures preserve draft/evidence and explicit review. Provider-specific errors remain mocked; no live reachability proof. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Stale snapshot is rejected without overwriting the newer draft. Explicit multi-chat recovery no longer locks out both conversations. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
+      </x:c>
+      <x:c r="S108" s="17" t="str">
+        <x:v>Only the creation transaction/reload/retry path was fixed and tested in this batch. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T108" s="1"/>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
@@ -6067,9 +6674,15 @@
       <x:c r="P109" s="19" t="str">
         <x:v>Performance check not run; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q109" s="1"/>
-      <x:c r="R109" s="1"/>
-      <x:c r="S109" s="1"/>
+      <x:c r="Q109" s="19" t="str">
+        <x:v>Unverified</x:v>
+      </x:c>
+      <x:c r="R109" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S109" s="19" t="str">
+        <x:v>A browser-control timeout occurred on the live artifact view; cause was not isolated and is not counted as a product defect. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T109" s="1"/>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
@@ -6121,9 +6734,15 @@
       <x:c r="P110" s="17" t="str">
         <x:v>A0; polished.js initialization; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q110" s="1"/>
-      <x:c r="R110" s="1"/>
-      <x:c r="S110" s="1"/>
+      <x:c r="Q110" s="17" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R110" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S110" s="17" t="str">
+        <x:v>Provider/device readiness and selected device are not part of onboarding. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T110" s="1"/>
     </x:row>
     <x:row r="111" ht="177" customHeight="1">
@@ -6175,9 +6794,15 @@
       <x:c r="P111" s="19" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/runtime/verify-backup-schema.cjs:4-28 (current six backup/transaction/size tests); .intentgraph/evidence/ux-fixes-2026-09-15/local-data-ui.json (roundtrip/Add/replace/reload); .intentgraph/evidence/ux-fixes-2026-09-15/history-regression.json (revert/avatar/history) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q111" s="1"/>
-      <x:c r="R111" s="1"/>
-      <x:c r="S111" s="1"/>
+      <x:c r="Q111" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R111" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S111" s="19" t="str">
+        <x:v>It did not prove exact migration preservation of all chats, drafts, queues, avatars and revert history. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T111" s="1"/>
     </x:row>
     <x:row r="112" ht="87" customHeight="1">
@@ -6229,9 +6854,15 @@
       <x:c r="P112" s="17" t="str">
         <x:v>2026-09-16: diagnostics-ui.json; verify-chat-read-api.cjs. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q112" s="1"/>
-      <x:c r="R112" s="1"/>
-      <x:c r="S112" s="1"/>
+      <x:c r="Q112" s="17" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R112" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S112" s="17" t="str">
+        <x:v>Local status fixtures and served build identity only; no live provider/device reachability claim. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T112" s="1"/>
     </x:row>
     <x:row r="113" ht="117" customHeight="1">
@@ -6283,9 +6914,15 @@
       <x:c r="P113" s="19" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q113" s="1"/>
-      <x:c r="R113" s="1"/>
-      <x:c r="S113" s="1"/>
+      <x:c r="Q113" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R113" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S113" s="19" t="str">
+        <x:v>The known rename inconsistency is resolved; complete terminology and icon acceptance is not yet verified. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T113" s="1"/>
     </x:row>
     <x:row r="114" ht="42" customHeight="1">
@@ -6337,9 +6974,15 @@
       <x:c r="P114" s="17" t="str">
         <x:v>architecture.json; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q114" s="1"/>
-      <x:c r="R114" s="1"/>
-      <x:c r="S114" s="1"/>
+      <x:c r="Q114" s="17" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="R114" s="17" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S114" s="17" t="str">
+        <x:v>Deferred by user decision. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T114" s="1"/>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
@@ -6391,9 +7034,15 @@
       <x:c r="P115" s="19" t="str">
         <x:v>User feedback; current audit; polished.css:45-64,116-143,325-329; polished.js:19-58,437-449</x:v>
       </x:c>
-      <x:c r="Q115" s="1"/>
-      <x:c r="R115" s="1"/>
-      <x:c r="S115" s="1"/>
+      <x:c r="Q115" s="19" t="str">
+        <x:v>Unverified</x:v>
+      </x:c>
+      <x:c r="R115" s="19" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S115" s="19" t="str">
+        <x:v>Owner acceptance unavailable. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T115" s="1"/>
     </x:row>
     <x:row r="116" ht="132" customHeight="1">
@@ -6445,9 +7094,15 @@
       <x:c r="P116" s="21" t="str">
         <x:v>2026-09-16: preservation audit PASS. 25/25 local fixture tests passed: agent-runtime/chat-runtime/network-execution/sandbox-routes/steering suites (allowlist, exact target, failed transport, read-only origin/header); no provider/device calls Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q116" s="1"/>
-      <x:c r="R116" s="1"/>
-      <x:c r="S116" s="1"/>
+      <x:c r="Q116" s="21" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R116" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S116" s="21" t="str">
+        <x:v>Local fixtures only; no provider/device calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T116" s="1"/>
     </x:row>
     <x:row r="117" ht="87" customHeight="1">
@@ -6499,9 +7154,15 @@
       <x:c r="P117" s="19" t="str">
         <x:v>2026-09-16: verify-queue-terminal.cjs 4/4; run-durability.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q117" s="1"/>
-      <x:c r="R117" s="1"/>
-      <x:c r="S117" s="1"/>
+      <x:c r="Q117" s="19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R117" s="19" t="str">
+        <x:v>Cancellation and dead-owner recovery remain UNKNOWN; replay and recovery cause no duplicate fixture responder invocation. No claim of stopping a remote device command. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.</x:v>
+      </x:c>
+      <x:c r="S117" s="19" t="str">
+        <x:v>Stop UX and duplicate-retry prevention were not freshly exercised; no provider/device calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T117" s="1"/>
     </x:row>
     <x:row r="118" ht="87" customHeight="1">
@@ -6553,9 +7214,15 @@
       <x:c r="P118" s="21" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/chat-interactions.json; verify-chat-interactions.cjs exit 0. Mocked requests; owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q118" s="1"/>
-      <x:c r="R118" s="1"/>
-      <x:c r="S118" s="1"/>
+      <x:c r="Q118" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R118" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S118" s="21" t="str">
+        <x:v>A fresh over-limit request/omission-count comparison was not completed. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T118" s="1"/>
     </x:row>
     <x:row r="119" ht="117" customHeight="1">
@@ -6607,9 +7274,15 @@
       <x:c r="P119" s="15" t="str">
         <x:v>2026-09-15: .intentgraph/evidence/ux-fixes-2026-09-15/{root-review.json,history-regression.json,reaction-recovery.json}; isolated browser checks exit 0. No provider/device calls; no physical-device or owner acceptance.</x:v>
       </x:c>
-      <x:c r="Q119" s="1"/>
-      <x:c r="R119" s="1"/>
-      <x:c r="S119" s="1"/>
+      <x:c r="Q119" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R119" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S119" s="15" t="str">
+        <x:v>This audit did not save a note and inspect the next model request to verify exclusion. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T119" s="1"/>
     </x:row>
     <x:row r="120" ht="87" customHeight="1">
@@ -6661,9 +7334,15 @@
       <x:c r="P120" s="21" t="str">
         <x:v>2026-09-15: edit-rendering.json and verify-edit-rendering.cjs exit 0 validate safe-link slice only. Full media acceptance remains pending.</x:v>
       </x:c>
-      <x:c r="Q120" s="1"/>
-      <x:c r="R120" s="1"/>
-      <x:c r="S120" s="1"/>
+      <x:c r="Q120" s="21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R120" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S120" s="21" t="str">
+        <x:v>Inline media and attachment reading remain pending. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T120" s="1"/>
     </x:row>
     <x:row r="121" ht="102" customHeight="1">
@@ -6715,9 +7394,15 @@
       <x:c r="P121" s="15" t="str">
         <x:v>2026-09-16: preservation audit PASS. .intentgraph/evidence/pending-88-20260916/preserved-audit.json (beforeOpen=true, afterOpen=false; no request path) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q121" s="1"/>
-      <x:c r="R121" s="1"/>
-      <x:c r="S121" s="1"/>
+      <x:c r="Q121" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R121" s="15" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S121" s="15" t="str">
+        <x:v>All exercised browser-local unread/reload/open and held local-run switching checks pass; provider execution and assistive-technology coverage remain outside this review. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T121" s="1"/>
     </x:row>
     <x:row r="122" ht="72" customHeight="1">
@@ -6769,9 +7454,15 @@
       <x:c r="P122" s="21" t="str">
         <x:v>2026-09-16: diagnostics-ui.json. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q122" s="1"/>
-      <x:c r="R122" s="1"/>
-      <x:c r="S122" s="1"/>
+      <x:c r="Q122" s="21" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R122" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S122" s="21" t="str">
+        <x:v>English fallback and disabled unsupported-language disclosure pass; additional translation coverage remains outside this review. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T122" s="1"/>
     </x:row>
     <x:row r="123" ht="87" customHeight="1">
@@ -6823,9 +7514,16 @@
       <x:c r="P123" s="15" t="str">
         <x:v>2026-09-16: alerts.json; verify-queue-terminal.cjs 4/4. Isolated tests passed; no live provider/device call. Owner acceptance pending.</x:v>
       </x:c>
-      <x:c r="Q123" s="1"/>
-      <x:c r="R123" s="1"/>
-      <x:c r="S123" s="1"/>
+      <x:c r="Q123" s="15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="R123" s="15" t="str">
+        <x:v>Active API enforces serial capacity; current browser waiting/draft fixture and queue checks supplement prior evidence. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: A genuinely live other-tab writer retains its Web Lock and completes successfully; foreign review is read-only until it finishes. Global backend serial admission remains. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
+      </x:c>
+      <x:c r="S123" s="15" t="str">
+        <x:v>Full serial multi-conversation queue UI was not exercised in this bounded run. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone. Browser admission writes require Web Locks; Windows remains unverified.</x:v>
+      </x:c>
       <x:c r="T123" s="1"/>
     </x:row>
     <x:row r="124" ht="42" customHeight="1">
@@ -6877,9 +7575,15 @@
       <x:c r="P124" s="21" t="str">
         <x:v>intentgraph/ui/index.html:7-8; adapters/index.cjs:462-503,570-598</x:v>
       </x:c>
-      <x:c r="Q124" s="1"/>
-      <x:c r="R124" s="1"/>
-      <x:c r="S124" s="1"/>
+      <x:c r="Q124" s="21" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="R124" s="21" t="str">
+        <x:v>No fresh acceptance run in this milestone; inherited dated effective evidence.</x:v>
+      </x:c>
+      <x:c r="S124" s="21" t="str">
+        <x:v>Local fixtures only; no provider/device calls. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T124" s="1"/>
     </x:row>
     <x:row r="125" ht="132" customHeight="1">
@@ -6931,9 +7635,16 @@
       <x:c r="P125" s="15" t="str">
         <x:v>2026-09-16: preservation audit PASS. isolated `verify-chat-read-api.cjs` passed (original raw provenance/read-back; secret fields stripped); .intentgraph/evidence/pending-88-20260916/run-recovery.json (reload/deep links/durable capture) Owner acceptance remains separate.</x:v>
       </x:c>
-      <x:c r="Q125" s="1"/>
-      <x:c r="R125" s="1"/>
-      <x:c r="S125" s="1"/>
+      <x:c r="Q125" s="15" t="str">
+        <x:v>Verified (scoped)</x:v>
+      </x:c>
+      <x:c r="R125" s="15" t="str">
+        <x:v>Current scoped receipt and raw-run readback preserve original run/request/chat provenance and exact output. Evidence and admission settlement are distinct. Evidence: docs/evidence/admission-2026-09-19/verification.json; browser-checks.json.
+Review correction: Captured event/evidence payloads survive reconciliation; repeated identical capture entries are deduplicated. Evidence-versus-receipt ambiguity remains a nonblocking limitation. Evidence: docs/evidence/admission-2026-09-19/review-fixes/verification.json</x:v>
+      </x:c>
+      <x:c r="S125" s="15" t="str">
+        <x:v>Existing local records only; no new provider/device run, service restart or cross-device durability test. Windows behavior, owner UI approval and live provider/device acceptance are not established by this milestone.</x:v>
+      </x:c>
       <x:c r="T125" s="1"/>
     </x:row>
     <x:row r="126">
@@ -7767,7 +8478,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b91acc2d02d4683"/>
+    <x:tablePart ns1:id="R3b91acc2d02d4683"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>